<commit_message>
fix: restaurar templates originales de logimat e imcdep
Los templates fueron modificados en commit 33385b4 para soportar el
enfoque de insert_rows, que luego fue revertido. Los templates modificados
son incompatibles con la escritura directa de celdas usada actualmente.

Se restauran los templates al estado anterior a fac0a3d (commit d8f8d3c).
También se corrige el nombre del logo en logimat/config.json
(logo_logimat.png, no logimat_logo.png).
</commit_message>
<xml_diff>
--- a/backend/app/platforms/imcdep/template.xlsx
+++ b/backend/app/platforms/imcdep/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zymo-intranet\backend\app\platforms\imcdep\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zymo-intranet\claude\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00E8DBC8-EF62-4F27-8B35-48E651D93465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C6C813F-6468-4D94-ABA9-0D0771196749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-620" windowWidth="19420" windowHeight="11500" xr2:uid="{5F00901D-42B5-4F93-81A8-46501A5E9861}"/>
+    <workbookView xWindow="2350" yWindow="1630" windowWidth="14400" windowHeight="8170" xr2:uid="{5F00901D-42B5-4F93-81A8-46501A5E9861}"/>
   </bookViews>
   <sheets>
     <sheet name="IMC DEPOSITO" sheetId="2" r:id="rId1"/>
@@ -1044,12 +1044,54 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1065,12 +1107,72 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1087,11 +1189,26 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1113,8 +1230,20 @@
     <xf numFmtId="167" fontId="20" fillId="0" borderId="30" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="20" fillId="0" borderId="33" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="21" fillId="2" borderId="34" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1126,6 +1255,30 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1159,218 +1312,65 @@
     <xf numFmtId="169" fontId="28" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="28" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="28" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="28" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="28" fillId="0" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1401,7 +1401,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>96</xdr:row>
+      <xdr:row>93</xdr:row>
       <xdr:rowOff>28576</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="0" cy="163166"/>
@@ -1447,7 +1447,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>112058</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>46504</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="0" cy="602689"/>
@@ -1875,21 +1875,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD0B5DA2-12C2-4D26-8CEB-4113728014FE}">
-  <dimension ref="A1:IV48"/>
+  <dimension ref="A1:IV45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="13.5" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="3" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" style="1" customWidth="1"/>
-    <col min="6" max="6" width="47.42578125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="16.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="47.36328125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="16.81640625" style="1" customWidth="1"/>
     <col min="9" max="10" width="3" style="1" customWidth="1"/>
     <col min="11" max="256" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="257" max="16384" width="10.7109375" style="1" hidden="1"/>
+    <col min="257" max="16384" width="10.7265625" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.25">
+    <row r="1" spans="1:256" ht="14">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1901,7 +1901,7 @@
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:11" ht="15" thickBot="1">
+    <row r="2" spans="1:256" ht="14.5" thickBot="1">
       <c r="A2" s="3"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -1913,1015 +1913,1752 @@
       <c r="I2" s="4"/>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:11" ht="21">
+    <row r="3" spans="1:256" ht="21">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
-      <c r="C3" s="101" t="e" vm="1">
+      <c r="C3" s="116" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="D3" s="102"/>
-      <c r="E3" s="105" t="s">
+      <c r="D3" s="115"/>
+      <c r="E3" s="114" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="105"/>
-      <c r="G3" s="105"/>
-      <c r="H3" s="106"/>
+      <c r="F3" s="114"/>
+      <c r="G3" s="114"/>
+      <c r="H3" s="113"/>
       <c r="I3" s="4"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:11" ht="18.399999999999999" customHeight="1">
+    <row r="4" spans="1:256" ht="18.399999999999999" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
-      <c r="C4" s="103"/>
-      <c r="D4" s="104"/>
-      <c r="E4" s="49" t="s">
+      <c r="C4" s="107"/>
+      <c r="D4" s="106"/>
+      <c r="E4" s="112" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="48" t="s">
+      <c r="F4" s="111" t="s">
         <v>52</v>
       </c>
-      <c r="G4" s="107" t="s">
+      <c r="G4" s="110" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="108"/>
+      <c r="H4" s="109"/>
       <c r="I4" s="4"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:11" ht="18.399999999999999" customHeight="1">
+    <row r="5" spans="1:256" ht="18.399999999999999" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
-      <c r="C5" s="103"/>
-      <c r="D5" s="104"/>
-      <c r="E5" s="47" t="s">
+      <c r="C5" s="107"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="108" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="109">
+      <c r="F5" s="104">
         <v>46084</v>
       </c>
-      <c r="G5" s="109"/>
-      <c r="H5" s="110"/>
+      <c r="G5" s="104"/>
+      <c r="H5" s="103"/>
       <c r="I5" s="4"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:11" ht="18.399999999999999" customHeight="1">
+    <row r="6" spans="1:256" ht="18.399999999999999" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="46" t="s">
+      <c r="C6" s="107"/>
+      <c r="D6" s="106"/>
+      <c r="E6" s="105" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="109" t="s">
+      <c r="F6" s="104" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="109"/>
-      <c r="H6" s="110"/>
+      <c r="G6" s="104"/>
+      <c r="H6" s="103"/>
       <c r="I6" s="4"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:11" ht="18.399999999999999" customHeight="1">
+    <row r="7" spans="1:256" ht="18.399999999999999" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
-      <c r="C7" s="103"/>
-      <c r="D7" s="104"/>
-      <c r="E7" s="46" t="s">
+      <c r="C7" s="107"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="105" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="109" t="s">
+      <c r="F7" s="104" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="109"/>
-      <c r="H7" s="110"/>
+      <c r="G7" s="104"/>
+      <c r="H7" s="103"/>
       <c r="I7" s="4"/>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:11" ht="18.399999999999999" customHeight="1">
+    <row r="8" spans="1:256" ht="18.399999999999999" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
-      <c r="C8" s="111" t="s">
+      <c r="C8" s="102" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="112"/>
-      <c r="E8" s="112"/>
-      <c r="F8" s="113" t="s">
+      <c r="D8" s="101"/>
+      <c r="E8" s="101"/>
+      <c r="F8" s="100" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="113"/>
-      <c r="H8" s="114"/>
+      <c r="G8" s="100"/>
+      <c r="H8" s="99"/>
       <c r="I8" s="4"/>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="44.1" customHeight="1" thickBot="1">
+    <row r="9" spans="1:256" ht="44" customHeight="1" thickBot="1">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
-      <c r="C9" s="115" t="s">
+      <c r="C9" s="98" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="116"/>
-      <c r="E9" s="116"/>
-      <c r="F9" s="45" t="s">
+      <c r="D9" s="97"/>
+      <c r="E9" s="97"/>
+      <c r="F9" s="96" t="s">
         <v>42</v>
       </c>
-      <c r="G9" s="45" t="s">
+      <c r="G9" s="96" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="44">
+      <c r="H9" s="95">
         <v>279901</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:11" ht="30">
+    <row r="10" spans="1:256" ht="14.5">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="94" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="42" t="s">
+      <c r="D10" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="93" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="41" t="s">
+      <c r="G10" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="40" t="s">
+      <c r="H10" s="91" t="s">
         <v>28</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="3"/>
-      <c r="K10" s="35"/>
+      <c r="K10" s="86"/>
     </row>
-    <row r="11" spans="1:11" ht="15">
+    <row r="11" spans="1:256" ht="14.5">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="39">
+      <c r="C11" s="90">
         <v>1</v>
       </c>
-      <c r="D11" s="39">
+      <c r="D11" s="90">
         <v>1</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="38" t="s">
+      <c r="E11" s="90"/>
+      <c r="F11" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="37">
+      <c r="G11" s="88">
         <v>60720.19</v>
       </c>
-      <c r="H11" s="36">
+      <c r="H11" s="87">
         <f>+G11*D11</f>
         <v>60720.19</v>
       </c>
       <c r="I11" s="4"/>
       <c r="J11" s="3"/>
-      <c r="K11" s="35"/>
+      <c r="K11" s="86"/>
     </row>
-    <row r="12" spans="1:11" ht="15">
+    <row r="12" spans="1:256" ht="21" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="36"/>
+      <c r="C12" s="85" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="84"/>
+      <c r="E12" s="84"/>
+      <c r="F12" s="84"/>
+      <c r="G12" s="84"/>
+      <c r="H12" s="83"/>
       <c r="I12" s="4"/>
       <c r="J12" s="3"/>
-      <c r="K12" s="35"/>
+      <c r="K12" s="74"/>
     </row>
-    <row r="13" spans="1:11" ht="15">
+    <row r="13" spans="1:256" ht="59.25" customHeight="1" thickBot="1">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="36"/>
+      <c r="C13" s="82" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="81"/>
+      <c r="E13" s="81"/>
+      <c r="F13" s="81"/>
+      <c r="G13" s="81"/>
+      <c r="H13" s="80"/>
       <c r="I13" s="4"/>
       <c r="J13" s="3"/>
-      <c r="K13" s="35"/>
+      <c r="K13" s="74"/>
     </row>
-    <row r="14" spans="1:11" ht="15">
+    <row r="14" spans="1:256" ht="21">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="36"/>
+      <c r="C14" s="79" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="78"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="77" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="76"/>
+      <c r="H14" s="75"/>
       <c r="I14" s="4"/>
       <c r="J14" s="3"/>
-      <c r="K14" s="35"/>
+      <c r="K14" s="74"/>
     </row>
-    <row r="15" spans="1:11" ht="21" customHeight="1">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="89" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="90"/>
-      <c r="E15" s="90"/>
-      <c r="F15" s="90"/>
-      <c r="G15" s="90"/>
-      <c r="H15" s="91"/>
+    <row r="15" spans="1:256" s="5" customFormat="1" ht="14.5">
+      <c r="A15" s="6"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="73" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
+      <c r="F15" s="72"/>
+      <c r="G15" s="72"/>
+      <c r="H15" s="71">
+        <f>SUM(H11:H11)</f>
+        <v>60720.19</v>
+      </c>
       <c r="I15" s="4"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="31"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="1"/>
+      <c r="W15" s="1"/>
+      <c r="X15" s="1"/>
+      <c r="Y15" s="1"/>
+      <c r="Z15" s="1"/>
+      <c r="AA15" s="1"/>
+      <c r="AB15" s="1"/>
+      <c r="AC15" s="1"/>
+      <c r="AD15" s="1"/>
+      <c r="AE15" s="1"/>
+      <c r="AF15" s="1"/>
+      <c r="AG15" s="1"/>
+      <c r="AH15" s="1"/>
+      <c r="AI15" s="1"/>
+      <c r="AJ15" s="1"/>
+      <c r="AK15" s="1"/>
+      <c r="AL15" s="1"/>
+      <c r="AM15" s="1"/>
+      <c r="AN15" s="1"/>
+      <c r="AO15" s="1"/>
+      <c r="AP15" s="1"/>
+      <c r="AQ15" s="1"/>
+      <c r="AR15" s="1"/>
+      <c r="AS15" s="1"/>
+      <c r="AT15" s="1"/>
+      <c r="AU15" s="1"/>
+      <c r="AV15" s="1"/>
+      <c r="AW15" s="1"/>
+      <c r="AX15" s="1"/>
+      <c r="AY15" s="1"/>
+      <c r="AZ15" s="1"/>
+      <c r="BA15" s="1"/>
+      <c r="BB15" s="1"/>
+      <c r="BC15" s="1"/>
+      <c r="BD15" s="1"/>
+      <c r="BE15" s="1"/>
+      <c r="BF15" s="1"/>
+      <c r="BG15" s="1"/>
+      <c r="BH15" s="1"/>
+      <c r="BI15" s="1"/>
+      <c r="BJ15" s="1"/>
+      <c r="BK15" s="1"/>
+      <c r="BL15" s="1"/>
+      <c r="BM15" s="1"/>
+      <c r="BN15" s="1"/>
+      <c r="BO15" s="1"/>
+      <c r="BP15" s="1"/>
+      <c r="BQ15" s="1"/>
+      <c r="BR15" s="1"/>
+      <c r="BS15" s="1"/>
+      <c r="BT15" s="1"/>
+      <c r="BU15" s="1"/>
+      <c r="BV15" s="1"/>
+      <c r="BW15" s="1"/>
+      <c r="BX15" s="1"/>
+      <c r="BY15" s="1"/>
+      <c r="BZ15" s="1"/>
+      <c r="CA15" s="1"/>
+      <c r="CB15" s="1"/>
+      <c r="CC15" s="1"/>
+      <c r="CD15" s="1"/>
+      <c r="CE15" s="1"/>
+      <c r="CF15" s="1"/>
+      <c r="CG15" s="1"/>
+      <c r="CH15" s="1"/>
+      <c r="CI15" s="1"/>
+      <c r="CJ15" s="1"/>
+      <c r="CK15" s="1"/>
+      <c r="CL15" s="1"/>
+      <c r="CM15" s="1"/>
+      <c r="CN15" s="1"/>
+      <c r="CO15" s="1"/>
+      <c r="CP15" s="1"/>
+      <c r="CQ15" s="1"/>
+      <c r="CR15" s="1"/>
+      <c r="CS15" s="1"/>
+      <c r="CT15" s="1"/>
+      <c r="CU15" s="1"/>
+      <c r="CV15" s="1"/>
+      <c r="CW15" s="1"/>
+      <c r="CX15" s="1"/>
+      <c r="CY15" s="1"/>
+      <c r="CZ15" s="1"/>
+      <c r="DA15" s="1"/>
+      <c r="DB15" s="1"/>
+      <c r="DC15" s="1"/>
+      <c r="DD15" s="1"/>
+      <c r="DE15" s="1"/>
+      <c r="DF15" s="1"/>
+      <c r="DG15" s="1"/>
+      <c r="DH15" s="1"/>
+      <c r="DI15" s="1"/>
+      <c r="DJ15" s="1"/>
+      <c r="DK15" s="1"/>
+      <c r="DL15" s="1"/>
+      <c r="DM15" s="1"/>
+      <c r="DN15" s="1"/>
+      <c r="DO15" s="1"/>
+      <c r="DP15" s="1"/>
+      <c r="DQ15" s="1"/>
+      <c r="DR15" s="1"/>
+      <c r="DS15" s="1"/>
+      <c r="DT15" s="1"/>
+      <c r="DU15" s="1"/>
+      <c r="DV15" s="1"/>
+      <c r="DW15" s="1"/>
+      <c r="DX15" s="1"/>
+      <c r="DY15" s="1"/>
+      <c r="DZ15" s="1"/>
+      <c r="EA15" s="1"/>
+      <c r="EB15" s="1"/>
+      <c r="EC15" s="1"/>
+      <c r="ED15" s="1"/>
+      <c r="EE15" s="1"/>
+      <c r="EF15" s="1"/>
+      <c r="EG15" s="1"/>
+      <c r="EH15" s="1"/>
+      <c r="EI15" s="1"/>
+      <c r="EJ15" s="1"/>
+      <c r="EK15" s="1"/>
+      <c r="EL15" s="1"/>
+      <c r="EM15" s="1"/>
+      <c r="EN15" s="1"/>
+      <c r="EO15" s="1"/>
+      <c r="EP15" s="1"/>
+      <c r="EQ15" s="1"/>
+      <c r="ER15" s="1"/>
+      <c r="ES15" s="1"/>
+      <c r="ET15" s="1"/>
+      <c r="EU15" s="1"/>
+      <c r="EV15" s="1"/>
+      <c r="EW15" s="1"/>
+      <c r="EX15" s="1"/>
+      <c r="EY15" s="1"/>
+      <c r="EZ15" s="1"/>
+      <c r="FA15" s="1"/>
+      <c r="FB15" s="1"/>
+      <c r="FC15" s="1"/>
+      <c r="FD15" s="1"/>
+      <c r="FE15" s="1"/>
+      <c r="FF15" s="1"/>
+      <c r="FG15" s="1"/>
+      <c r="FH15" s="1"/>
+      <c r="FI15" s="1"/>
+      <c r="FJ15" s="1"/>
+      <c r="FK15" s="1"/>
+      <c r="FL15" s="1"/>
+      <c r="FM15" s="1"/>
+      <c r="FN15" s="1"/>
+      <c r="FO15" s="1"/>
+      <c r="FP15" s="1"/>
+      <c r="FQ15" s="1"/>
+      <c r="FR15" s="1"/>
+      <c r="FS15" s="1"/>
+      <c r="FT15" s="1"/>
+      <c r="FU15" s="1"/>
+      <c r="FV15" s="1"/>
+      <c r="FW15" s="1"/>
+      <c r="FX15" s="1"/>
+      <c r="FY15" s="1"/>
+      <c r="FZ15" s="1"/>
+      <c r="GA15" s="1"/>
+      <c r="GB15" s="1"/>
+      <c r="GC15" s="1"/>
+      <c r="GD15" s="1"/>
+      <c r="GE15" s="1"/>
+      <c r="GF15" s="1"/>
+      <c r="GG15" s="1"/>
+      <c r="GH15" s="1"/>
+      <c r="GI15" s="1"/>
+      <c r="GJ15" s="1"/>
+      <c r="GK15" s="1"/>
+      <c r="GL15" s="1"/>
+      <c r="GM15" s="1"/>
+      <c r="GN15" s="1"/>
+      <c r="GO15" s="1"/>
+      <c r="GP15" s="1"/>
+      <c r="GQ15" s="1"/>
+      <c r="GR15" s="1"/>
+      <c r="GS15" s="1"/>
+      <c r="GT15" s="1"/>
+      <c r="GU15" s="1"/>
+      <c r="GV15" s="1"/>
+      <c r="GW15" s="1"/>
+      <c r="GX15" s="1"/>
+      <c r="GY15" s="1"/>
+      <c r="GZ15" s="1"/>
+      <c r="HA15" s="1"/>
+      <c r="HB15" s="1"/>
+      <c r="HC15" s="1"/>
+      <c r="HD15" s="1"/>
+      <c r="HE15" s="1"/>
+      <c r="HF15" s="1"/>
+      <c r="HG15" s="1"/>
+      <c r="HH15" s="1"/>
+      <c r="HI15" s="1"/>
+      <c r="HJ15" s="1"/>
+      <c r="HK15" s="1"/>
+      <c r="HL15" s="1"/>
+      <c r="HM15" s="1"/>
+      <c r="HN15" s="1"/>
+      <c r="HO15" s="1"/>
+      <c r="HP15" s="1"/>
+      <c r="HQ15" s="1"/>
+      <c r="HR15" s="1"/>
+      <c r="HS15" s="1"/>
+      <c r="HT15" s="1"/>
+      <c r="HU15" s="1"/>
+      <c r="HV15" s="1"/>
+      <c r="HW15" s="1"/>
+      <c r="HX15" s="1"/>
+      <c r="HY15" s="1"/>
+      <c r="HZ15" s="1"/>
+      <c r="IA15" s="1"/>
+      <c r="IB15" s="1"/>
+      <c r="IC15" s="1"/>
+      <c r="ID15" s="1"/>
+      <c r="IE15" s="1"/>
+      <c r="IF15" s="1"/>
+      <c r="IG15" s="1"/>
+      <c r="IH15" s="1"/>
+      <c r="II15" s="1"/>
+      <c r="IJ15" s="1"/>
+      <c r="IK15" s="1"/>
+      <c r="IL15" s="1"/>
+      <c r="IM15" s="1"/>
+      <c r="IN15" s="1"/>
+      <c r="IO15" s="1"/>
+      <c r="IP15" s="1"/>
+      <c r="IQ15" s="1"/>
+      <c r="IR15" s="1"/>
+      <c r="IS15" s="1"/>
+      <c r="IT15" s="1"/>
+      <c r="IU15" s="1"/>
+      <c r="IV15" s="1"/>
     </row>
-    <row r="16" spans="1:11" ht="59.25" customHeight="1" thickBot="1">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="93"/>
-      <c r="E16" s="93"/>
-      <c r="F16" s="93"/>
-      <c r="G16" s="93"/>
-      <c r="H16" s="94"/>
+    <row r="16" spans="1:256" s="5" customFormat="1" ht="14.5">
+      <c r="A16" s="6"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="73" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="72"/>
+      <c r="E16" s="72"/>
+      <c r="F16" s="72"/>
+      <c r="G16" s="72"/>
+      <c r="H16" s="71"/>
       <c r="I16" s="4"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="31"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="1"/>
+      <c r="W16" s="1"/>
+      <c r="X16" s="1"/>
+      <c r="Y16" s="1"/>
+      <c r="Z16" s="1"/>
+      <c r="AA16" s="1"/>
+      <c r="AB16" s="1"/>
+      <c r="AC16" s="1"/>
+      <c r="AD16" s="1"/>
+      <c r="AE16" s="1"/>
+      <c r="AF16" s="1"/>
+      <c r="AG16" s="1"/>
+      <c r="AH16" s="1"/>
+      <c r="AI16" s="1"/>
+      <c r="AJ16" s="1"/>
+      <c r="AK16" s="1"/>
+      <c r="AL16" s="1"/>
+      <c r="AM16" s="1"/>
+      <c r="AN16" s="1"/>
+      <c r="AO16" s="1"/>
+      <c r="AP16" s="1"/>
+      <c r="AQ16" s="1"/>
+      <c r="AR16" s="1"/>
+      <c r="AS16" s="1"/>
+      <c r="AT16" s="1"/>
+      <c r="AU16" s="1"/>
+      <c r="AV16" s="1"/>
+      <c r="AW16" s="1"/>
+      <c r="AX16" s="1"/>
+      <c r="AY16" s="1"/>
+      <c r="AZ16" s="1"/>
+      <c r="BA16" s="1"/>
+      <c r="BB16" s="1"/>
+      <c r="BC16" s="1"/>
+      <c r="BD16" s="1"/>
+      <c r="BE16" s="1"/>
+      <c r="BF16" s="1"/>
+      <c r="BG16" s="1"/>
+      <c r="BH16" s="1"/>
+      <c r="BI16" s="1"/>
+      <c r="BJ16" s="1"/>
+      <c r="BK16" s="1"/>
+      <c r="BL16" s="1"/>
+      <c r="BM16" s="1"/>
+      <c r="BN16" s="1"/>
+      <c r="BO16" s="1"/>
+      <c r="BP16" s="1"/>
+      <c r="BQ16" s="1"/>
+      <c r="BR16" s="1"/>
+      <c r="BS16" s="1"/>
+      <c r="BT16" s="1"/>
+      <c r="BU16" s="1"/>
+      <c r="BV16" s="1"/>
+      <c r="BW16" s="1"/>
+      <c r="BX16" s="1"/>
+      <c r="BY16" s="1"/>
+      <c r="BZ16" s="1"/>
+      <c r="CA16" s="1"/>
+      <c r="CB16" s="1"/>
+      <c r="CC16" s="1"/>
+      <c r="CD16" s="1"/>
+      <c r="CE16" s="1"/>
+      <c r="CF16" s="1"/>
+      <c r="CG16" s="1"/>
+      <c r="CH16" s="1"/>
+      <c r="CI16" s="1"/>
+      <c r="CJ16" s="1"/>
+      <c r="CK16" s="1"/>
+      <c r="CL16" s="1"/>
+      <c r="CM16" s="1"/>
+      <c r="CN16" s="1"/>
+      <c r="CO16" s="1"/>
+      <c r="CP16" s="1"/>
+      <c r="CQ16" s="1"/>
+      <c r="CR16" s="1"/>
+      <c r="CS16" s="1"/>
+      <c r="CT16" s="1"/>
+      <c r="CU16" s="1"/>
+      <c r="CV16" s="1"/>
+      <c r="CW16" s="1"/>
+      <c r="CX16" s="1"/>
+      <c r="CY16" s="1"/>
+      <c r="CZ16" s="1"/>
+      <c r="DA16" s="1"/>
+      <c r="DB16" s="1"/>
+      <c r="DC16" s="1"/>
+      <c r="DD16" s="1"/>
+      <c r="DE16" s="1"/>
+      <c r="DF16" s="1"/>
+      <c r="DG16" s="1"/>
+      <c r="DH16" s="1"/>
+      <c r="DI16" s="1"/>
+      <c r="DJ16" s="1"/>
+      <c r="DK16" s="1"/>
+      <c r="DL16" s="1"/>
+      <c r="DM16" s="1"/>
+      <c r="DN16" s="1"/>
+      <c r="DO16" s="1"/>
+      <c r="DP16" s="1"/>
+      <c r="DQ16" s="1"/>
+      <c r="DR16" s="1"/>
+      <c r="DS16" s="1"/>
+      <c r="DT16" s="1"/>
+      <c r="DU16" s="1"/>
+      <c r="DV16" s="1"/>
+      <c r="DW16" s="1"/>
+      <c r="DX16" s="1"/>
+      <c r="DY16" s="1"/>
+      <c r="DZ16" s="1"/>
+      <c r="EA16" s="1"/>
+      <c r="EB16" s="1"/>
+      <c r="EC16" s="1"/>
+      <c r="ED16" s="1"/>
+      <c r="EE16" s="1"/>
+      <c r="EF16" s="1"/>
+      <c r="EG16" s="1"/>
+      <c r="EH16" s="1"/>
+      <c r="EI16" s="1"/>
+      <c r="EJ16" s="1"/>
+      <c r="EK16" s="1"/>
+      <c r="EL16" s="1"/>
+      <c r="EM16" s="1"/>
+      <c r="EN16" s="1"/>
+      <c r="EO16" s="1"/>
+      <c r="EP16" s="1"/>
+      <c r="EQ16" s="1"/>
+      <c r="ER16" s="1"/>
+      <c r="ES16" s="1"/>
+      <c r="ET16" s="1"/>
+      <c r="EU16" s="1"/>
+      <c r="EV16" s="1"/>
+      <c r="EW16" s="1"/>
+      <c r="EX16" s="1"/>
+      <c r="EY16" s="1"/>
+      <c r="EZ16" s="1"/>
+      <c r="FA16" s="1"/>
+      <c r="FB16" s="1"/>
+      <c r="FC16" s="1"/>
+      <c r="FD16" s="1"/>
+      <c r="FE16" s="1"/>
+      <c r="FF16" s="1"/>
+      <c r="FG16" s="1"/>
+      <c r="FH16" s="1"/>
+      <c r="FI16" s="1"/>
+      <c r="FJ16" s="1"/>
+      <c r="FK16" s="1"/>
+      <c r="FL16" s="1"/>
+      <c r="FM16" s="1"/>
+      <c r="FN16" s="1"/>
+      <c r="FO16" s="1"/>
+      <c r="FP16" s="1"/>
+      <c r="FQ16" s="1"/>
+      <c r="FR16" s="1"/>
+      <c r="FS16" s="1"/>
+      <c r="FT16" s="1"/>
+      <c r="FU16" s="1"/>
+      <c r="FV16" s="1"/>
+      <c r="FW16" s="1"/>
+      <c r="FX16" s="1"/>
+      <c r="FY16" s="1"/>
+      <c r="FZ16" s="1"/>
+      <c r="GA16" s="1"/>
+      <c r="GB16" s="1"/>
+      <c r="GC16" s="1"/>
+      <c r="GD16" s="1"/>
+      <c r="GE16" s="1"/>
+      <c r="GF16" s="1"/>
+      <c r="GG16" s="1"/>
+      <c r="GH16" s="1"/>
+      <c r="GI16" s="1"/>
+      <c r="GJ16" s="1"/>
+      <c r="GK16" s="1"/>
+      <c r="GL16" s="1"/>
+      <c r="GM16" s="1"/>
+      <c r="GN16" s="1"/>
+      <c r="GO16" s="1"/>
+      <c r="GP16" s="1"/>
+      <c r="GQ16" s="1"/>
+      <c r="GR16" s="1"/>
+      <c r="GS16" s="1"/>
+      <c r="GT16" s="1"/>
+      <c r="GU16" s="1"/>
+      <c r="GV16" s="1"/>
+      <c r="GW16" s="1"/>
+      <c r="GX16" s="1"/>
+      <c r="GY16" s="1"/>
+      <c r="GZ16" s="1"/>
+      <c r="HA16" s="1"/>
+      <c r="HB16" s="1"/>
+      <c r="HC16" s="1"/>
+      <c r="HD16" s="1"/>
+      <c r="HE16" s="1"/>
+      <c r="HF16" s="1"/>
+      <c r="HG16" s="1"/>
+      <c r="HH16" s="1"/>
+      <c r="HI16" s="1"/>
+      <c r="HJ16" s="1"/>
+      <c r="HK16" s="1"/>
+      <c r="HL16" s="1"/>
+      <c r="HM16" s="1"/>
+      <c r="HN16" s="1"/>
+      <c r="HO16" s="1"/>
+      <c r="HP16" s="1"/>
+      <c r="HQ16" s="1"/>
+      <c r="HR16" s="1"/>
+      <c r="HS16" s="1"/>
+      <c r="HT16" s="1"/>
+      <c r="HU16" s="1"/>
+      <c r="HV16" s="1"/>
+      <c r="HW16" s="1"/>
+      <c r="HX16" s="1"/>
+      <c r="HY16" s="1"/>
+      <c r="HZ16" s="1"/>
+      <c r="IA16" s="1"/>
+      <c r="IB16" s="1"/>
+      <c r="IC16" s="1"/>
+      <c r="ID16" s="1"/>
+      <c r="IE16" s="1"/>
+      <c r="IF16" s="1"/>
+      <c r="IG16" s="1"/>
+      <c r="IH16" s="1"/>
+      <c r="II16" s="1"/>
+      <c r="IJ16" s="1"/>
+      <c r="IK16" s="1"/>
+      <c r="IL16" s="1"/>
+      <c r="IM16" s="1"/>
+      <c r="IN16" s="1"/>
+      <c r="IO16" s="1"/>
+      <c r="IP16" s="1"/>
+      <c r="IQ16" s="1"/>
+      <c r="IR16" s="1"/>
+      <c r="IS16" s="1"/>
+      <c r="IT16" s="1"/>
+      <c r="IU16" s="1"/>
+      <c r="IV16" s="1"/>
     </row>
-    <row r="17" spans="1:256" ht="21">
+    <row r="17" spans="1:256" ht="15" thickBot="1">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
-      <c r="C17" s="99" t="s">
-        <v>32</v>
-      </c>
-      <c r="D17" s="100"/>
-      <c r="E17" s="100"/>
-      <c r="F17" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="G17" s="33"/>
-      <c r="H17" s="32"/>
+      <c r="C17" s="70" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="69"/>
+      <c r="E17" s="69"/>
+      <c r="F17" s="69"/>
+      <c r="G17" s="69"/>
+      <c r="H17" s="68">
+        <f>H16+H15</f>
+        <v>60720.19</v>
+      </c>
       <c r="I17" s="4"/>
       <c r="J17" s="3"/>
-      <c r="K17" s="31"/>
     </row>
-    <row r="18" spans="1:256" s="5" customFormat="1" ht="15">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="95" t="s">
-        <v>30</v>
-      </c>
-      <c r="D18" s="96"/>
-      <c r="E18" s="96"/>
-      <c r="F18" s="96"/>
-      <c r="G18" s="96"/>
-      <c r="H18" s="30">
-        <f>SUM(H11:H11)</f>
-        <v>60720.19</v>
-      </c>
+    <row r="18" spans="1:256" ht="21.75" customHeight="1">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="67" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="65"/>
       <c r="I18" s="4"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="1"/>
-      <c r="U18" s="1"/>
-      <c r="V18" s="1"/>
-      <c r="W18" s="1"/>
-      <c r="X18" s="1"/>
-      <c r="Y18" s="1"/>
-      <c r="Z18" s="1"/>
-      <c r="AA18" s="1"/>
-      <c r="AB18" s="1"/>
-      <c r="AC18" s="1"/>
-      <c r="AD18" s="1"/>
-      <c r="AE18" s="1"/>
-      <c r="AF18" s="1"/>
-      <c r="AG18" s="1"/>
-      <c r="AH18" s="1"/>
-      <c r="AI18" s="1"/>
-      <c r="AJ18" s="1"/>
-      <c r="AK18" s="1"/>
-      <c r="AL18" s="1"/>
-      <c r="AM18" s="1"/>
-      <c r="AN18" s="1"/>
-      <c r="AO18" s="1"/>
-      <c r="AP18" s="1"/>
-      <c r="AQ18" s="1"/>
-      <c r="AR18" s="1"/>
-      <c r="AS18" s="1"/>
-      <c r="AT18" s="1"/>
-      <c r="AU18" s="1"/>
-      <c r="AV18" s="1"/>
-      <c r="AW18" s="1"/>
-      <c r="AX18" s="1"/>
-      <c r="AY18" s="1"/>
-      <c r="AZ18" s="1"/>
-      <c r="BA18" s="1"/>
-      <c r="BB18" s="1"/>
-      <c r="BC18" s="1"/>
-      <c r="BD18" s="1"/>
-      <c r="BE18" s="1"/>
-      <c r="BF18" s="1"/>
-      <c r="BG18" s="1"/>
-      <c r="BH18" s="1"/>
-      <c r="BI18" s="1"/>
-      <c r="BJ18" s="1"/>
-      <c r="BK18" s="1"/>
-      <c r="BL18" s="1"/>
-      <c r="BM18" s="1"/>
-      <c r="BN18" s="1"/>
-      <c r="BO18" s="1"/>
-      <c r="BP18" s="1"/>
-      <c r="BQ18" s="1"/>
-      <c r="BR18" s="1"/>
-      <c r="BS18" s="1"/>
-      <c r="BT18" s="1"/>
-      <c r="BU18" s="1"/>
-      <c r="BV18" s="1"/>
-      <c r="BW18" s="1"/>
-      <c r="BX18" s="1"/>
-      <c r="BY18" s="1"/>
-      <c r="BZ18" s="1"/>
-      <c r="CA18" s="1"/>
-      <c r="CB18" s="1"/>
-      <c r="CC18" s="1"/>
-      <c r="CD18" s="1"/>
-      <c r="CE18" s="1"/>
-      <c r="CF18" s="1"/>
-      <c r="CG18" s="1"/>
-      <c r="CH18" s="1"/>
-      <c r="CI18" s="1"/>
-      <c r="CJ18" s="1"/>
-      <c r="CK18" s="1"/>
-      <c r="CL18" s="1"/>
-      <c r="CM18" s="1"/>
-      <c r="CN18" s="1"/>
-      <c r="CO18" s="1"/>
-      <c r="CP18" s="1"/>
-      <c r="CQ18" s="1"/>
-      <c r="CR18" s="1"/>
-      <c r="CS18" s="1"/>
-      <c r="CT18" s="1"/>
-      <c r="CU18" s="1"/>
-      <c r="CV18" s="1"/>
-      <c r="CW18" s="1"/>
-      <c r="CX18" s="1"/>
-      <c r="CY18" s="1"/>
-      <c r="CZ18" s="1"/>
-      <c r="DA18" s="1"/>
-      <c r="DB18" s="1"/>
-      <c r="DC18" s="1"/>
-      <c r="DD18" s="1"/>
-      <c r="DE18" s="1"/>
-      <c r="DF18" s="1"/>
-      <c r="DG18" s="1"/>
-      <c r="DH18" s="1"/>
-      <c r="DI18" s="1"/>
-      <c r="DJ18" s="1"/>
-      <c r="DK18" s="1"/>
-      <c r="DL18" s="1"/>
-      <c r="DM18" s="1"/>
-      <c r="DN18" s="1"/>
-      <c r="DO18" s="1"/>
-      <c r="DP18" s="1"/>
-      <c r="DQ18" s="1"/>
-      <c r="DR18" s="1"/>
-      <c r="DS18" s="1"/>
-      <c r="DT18" s="1"/>
-      <c r="DU18" s="1"/>
-      <c r="DV18" s="1"/>
-      <c r="DW18" s="1"/>
-      <c r="DX18" s="1"/>
-      <c r="DY18" s="1"/>
-      <c r="DZ18" s="1"/>
-      <c r="EA18" s="1"/>
-      <c r="EB18" s="1"/>
-      <c r="EC18" s="1"/>
-      <c r="ED18" s="1"/>
-      <c r="EE18" s="1"/>
-      <c r="EF18" s="1"/>
-      <c r="EG18" s="1"/>
-      <c r="EH18" s="1"/>
-      <c r="EI18" s="1"/>
-      <c r="EJ18" s="1"/>
-      <c r="EK18" s="1"/>
-      <c r="EL18" s="1"/>
-      <c r="EM18" s="1"/>
-      <c r="EN18" s="1"/>
-      <c r="EO18" s="1"/>
-      <c r="EP18" s="1"/>
-      <c r="EQ18" s="1"/>
-      <c r="ER18" s="1"/>
-      <c r="ES18" s="1"/>
-      <c r="ET18" s="1"/>
-      <c r="EU18" s="1"/>
-      <c r="EV18" s="1"/>
-      <c r="EW18" s="1"/>
-      <c r="EX18" s="1"/>
-      <c r="EY18" s="1"/>
-      <c r="EZ18" s="1"/>
-      <c r="FA18" s="1"/>
-      <c r="FB18" s="1"/>
-      <c r="FC18" s="1"/>
-      <c r="FD18" s="1"/>
-      <c r="FE18" s="1"/>
-      <c r="FF18" s="1"/>
-      <c r="FG18" s="1"/>
-      <c r="FH18" s="1"/>
-      <c r="FI18" s="1"/>
-      <c r="FJ18" s="1"/>
-      <c r="FK18" s="1"/>
-      <c r="FL18" s="1"/>
-      <c r="FM18" s="1"/>
-      <c r="FN18" s="1"/>
-      <c r="FO18" s="1"/>
-      <c r="FP18" s="1"/>
-      <c r="FQ18" s="1"/>
-      <c r="FR18" s="1"/>
-      <c r="FS18" s="1"/>
-      <c r="FT18" s="1"/>
-      <c r="FU18" s="1"/>
-      <c r="FV18" s="1"/>
-      <c r="FW18" s="1"/>
-      <c r="FX18" s="1"/>
-      <c r="FY18" s="1"/>
-      <c r="FZ18" s="1"/>
-      <c r="GA18" s="1"/>
-      <c r="GB18" s="1"/>
-      <c r="GC18" s="1"/>
-      <c r="GD18" s="1"/>
-      <c r="GE18" s="1"/>
-      <c r="GF18" s="1"/>
-      <c r="GG18" s="1"/>
-      <c r="GH18" s="1"/>
-      <c r="GI18" s="1"/>
-      <c r="GJ18" s="1"/>
-      <c r="GK18" s="1"/>
-      <c r="GL18" s="1"/>
-      <c r="GM18" s="1"/>
-      <c r="GN18" s="1"/>
-      <c r="GO18" s="1"/>
-      <c r="GP18" s="1"/>
-      <c r="GQ18" s="1"/>
-      <c r="GR18" s="1"/>
-      <c r="GS18" s="1"/>
-      <c r="GT18" s="1"/>
-      <c r="GU18" s="1"/>
-      <c r="GV18" s="1"/>
-      <c r="GW18" s="1"/>
-      <c r="GX18" s="1"/>
-      <c r="GY18" s="1"/>
-      <c r="GZ18" s="1"/>
-      <c r="HA18" s="1"/>
-      <c r="HB18" s="1"/>
-      <c r="HC18" s="1"/>
-      <c r="HD18" s="1"/>
-      <c r="HE18" s="1"/>
-      <c r="HF18" s="1"/>
-      <c r="HG18" s="1"/>
-      <c r="HH18" s="1"/>
-      <c r="HI18" s="1"/>
-      <c r="HJ18" s="1"/>
-      <c r="HK18" s="1"/>
-      <c r="HL18" s="1"/>
-      <c r="HM18" s="1"/>
-      <c r="HN18" s="1"/>
-      <c r="HO18" s="1"/>
-      <c r="HP18" s="1"/>
-      <c r="HQ18" s="1"/>
-      <c r="HR18" s="1"/>
-      <c r="HS18" s="1"/>
-      <c r="HT18" s="1"/>
-      <c r="HU18" s="1"/>
-      <c r="HV18" s="1"/>
-      <c r="HW18" s="1"/>
-      <c r="HX18" s="1"/>
-      <c r="HY18" s="1"/>
-      <c r="HZ18" s="1"/>
-      <c r="IA18" s="1"/>
-      <c r="IB18" s="1"/>
-      <c r="IC18" s="1"/>
-      <c r="ID18" s="1"/>
-      <c r="IE18" s="1"/>
-      <c r="IF18" s="1"/>
-      <c r="IG18" s="1"/>
-      <c r="IH18" s="1"/>
-      <c r="II18" s="1"/>
-      <c r="IJ18" s="1"/>
-      <c r="IK18" s="1"/>
-      <c r="IL18" s="1"/>
-      <c r="IM18" s="1"/>
-      <c r="IN18" s="1"/>
-      <c r="IO18" s="1"/>
-      <c r="IP18" s="1"/>
-      <c r="IQ18" s="1"/>
-      <c r="IR18" s="1"/>
-      <c r="IS18" s="1"/>
-      <c r="IT18" s="1"/>
-      <c r="IU18" s="1"/>
-      <c r="IV18" s="1"/>
+      <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:256" s="5" customFormat="1" ht="15">
-      <c r="A19" s="6"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="95" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="96"/>
-      <c r="E19" s="96"/>
-      <c r="F19" s="96"/>
-      <c r="G19" s="96"/>
-      <c r="H19" s="30"/>
+    <row r="19" spans="1:256" ht="14.5">
+      <c r="A19" s="3"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="61" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="60"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="60"/>
+      <c r="G19" s="59" t="s">
+        <v>20</v>
+      </c>
+      <c r="H19" s="50"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
-      <c r="R19" s="1"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="1"/>
-      <c r="U19" s="1"/>
-      <c r="V19" s="1"/>
-      <c r="W19" s="1"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="1"/>
-      <c r="Z19" s="1"/>
-      <c r="AA19" s="1"/>
-      <c r="AB19" s="1"/>
-      <c r="AC19" s="1"/>
-      <c r="AD19" s="1"/>
-      <c r="AE19" s="1"/>
-      <c r="AF19" s="1"/>
-      <c r="AG19" s="1"/>
-      <c r="AH19" s="1"/>
-      <c r="AI19" s="1"/>
-      <c r="AJ19" s="1"/>
-      <c r="AK19" s="1"/>
-      <c r="AL19" s="1"/>
-      <c r="AM19" s="1"/>
-      <c r="AN19" s="1"/>
-      <c r="AO19" s="1"/>
-      <c r="AP19" s="1"/>
-      <c r="AQ19" s="1"/>
-      <c r="AR19" s="1"/>
-      <c r="AS19" s="1"/>
-      <c r="AT19" s="1"/>
-      <c r="AU19" s="1"/>
-      <c r="AV19" s="1"/>
-      <c r="AW19" s="1"/>
-      <c r="AX19" s="1"/>
-      <c r="AY19" s="1"/>
-      <c r="AZ19" s="1"/>
-      <c r="BA19" s="1"/>
-      <c r="BB19" s="1"/>
-      <c r="BC19" s="1"/>
-      <c r="BD19" s="1"/>
-      <c r="BE19" s="1"/>
-      <c r="BF19" s="1"/>
-      <c r="BG19" s="1"/>
-      <c r="BH19" s="1"/>
-      <c r="BI19" s="1"/>
-      <c r="BJ19" s="1"/>
-      <c r="BK19" s="1"/>
-      <c r="BL19" s="1"/>
-      <c r="BM19" s="1"/>
-      <c r="BN19" s="1"/>
-      <c r="BO19" s="1"/>
-      <c r="BP19" s="1"/>
-      <c r="BQ19" s="1"/>
-      <c r="BR19" s="1"/>
-      <c r="BS19" s="1"/>
-      <c r="BT19" s="1"/>
-      <c r="BU19" s="1"/>
-      <c r="BV19" s="1"/>
-      <c r="BW19" s="1"/>
-      <c r="BX19" s="1"/>
-      <c r="BY19" s="1"/>
-      <c r="BZ19" s="1"/>
-      <c r="CA19" s="1"/>
-      <c r="CB19" s="1"/>
-      <c r="CC19" s="1"/>
-      <c r="CD19" s="1"/>
-      <c r="CE19" s="1"/>
-      <c r="CF19" s="1"/>
-      <c r="CG19" s="1"/>
-      <c r="CH19" s="1"/>
-      <c r="CI19" s="1"/>
-      <c r="CJ19" s="1"/>
-      <c r="CK19" s="1"/>
-      <c r="CL19" s="1"/>
-      <c r="CM19" s="1"/>
-      <c r="CN19" s="1"/>
-      <c r="CO19" s="1"/>
-      <c r="CP19" s="1"/>
-      <c r="CQ19" s="1"/>
-      <c r="CR19" s="1"/>
-      <c r="CS19" s="1"/>
-      <c r="CT19" s="1"/>
-      <c r="CU19" s="1"/>
-      <c r="CV19" s="1"/>
-      <c r="CW19" s="1"/>
-      <c r="CX19" s="1"/>
-      <c r="CY19" s="1"/>
-      <c r="CZ19" s="1"/>
-      <c r="DA19" s="1"/>
-      <c r="DB19" s="1"/>
-      <c r="DC19" s="1"/>
-      <c r="DD19" s="1"/>
-      <c r="DE19" s="1"/>
-      <c r="DF19" s="1"/>
-      <c r="DG19" s="1"/>
-      <c r="DH19" s="1"/>
-      <c r="DI19" s="1"/>
-      <c r="DJ19" s="1"/>
-      <c r="DK19" s="1"/>
-      <c r="DL19" s="1"/>
-      <c r="DM19" s="1"/>
-      <c r="DN19" s="1"/>
-      <c r="DO19" s="1"/>
-      <c r="DP19" s="1"/>
-      <c r="DQ19" s="1"/>
-      <c r="DR19" s="1"/>
-      <c r="DS19" s="1"/>
-      <c r="DT19" s="1"/>
-      <c r="DU19" s="1"/>
-      <c r="DV19" s="1"/>
-      <c r="DW19" s="1"/>
-      <c r="DX19" s="1"/>
-      <c r="DY19" s="1"/>
-      <c r="DZ19" s="1"/>
-      <c r="EA19" s="1"/>
-      <c r="EB19" s="1"/>
-      <c r="EC19" s="1"/>
-      <c r="ED19" s="1"/>
-      <c r="EE19" s="1"/>
-      <c r="EF19" s="1"/>
-      <c r="EG19" s="1"/>
-      <c r="EH19" s="1"/>
-      <c r="EI19" s="1"/>
-      <c r="EJ19" s="1"/>
-      <c r="EK19" s="1"/>
-      <c r="EL19" s="1"/>
-      <c r="EM19" s="1"/>
-      <c r="EN19" s="1"/>
-      <c r="EO19" s="1"/>
-      <c r="EP19" s="1"/>
-      <c r="EQ19" s="1"/>
-      <c r="ER19" s="1"/>
-      <c r="ES19" s="1"/>
-      <c r="ET19" s="1"/>
-      <c r="EU19" s="1"/>
-      <c r="EV19" s="1"/>
-      <c r="EW19" s="1"/>
-      <c r="EX19" s="1"/>
-      <c r="EY19" s="1"/>
-      <c r="EZ19" s="1"/>
-      <c r="FA19" s="1"/>
-      <c r="FB19" s="1"/>
-      <c r="FC19" s="1"/>
-      <c r="FD19" s="1"/>
-      <c r="FE19" s="1"/>
-      <c r="FF19" s="1"/>
-      <c r="FG19" s="1"/>
-      <c r="FH19" s="1"/>
-      <c r="FI19" s="1"/>
-      <c r="FJ19" s="1"/>
-      <c r="FK19" s="1"/>
-      <c r="FL19" s="1"/>
-      <c r="FM19" s="1"/>
-      <c r="FN19" s="1"/>
-      <c r="FO19" s="1"/>
-      <c r="FP19" s="1"/>
-      <c r="FQ19" s="1"/>
-      <c r="FR19" s="1"/>
-      <c r="FS19" s="1"/>
-      <c r="FT19" s="1"/>
-      <c r="FU19" s="1"/>
-      <c r="FV19" s="1"/>
-      <c r="FW19" s="1"/>
-      <c r="FX19" s="1"/>
-      <c r="FY19" s="1"/>
-      <c r="FZ19" s="1"/>
-      <c r="GA19" s="1"/>
-      <c r="GB19" s="1"/>
-      <c r="GC19" s="1"/>
-      <c r="GD19" s="1"/>
-      <c r="GE19" s="1"/>
-      <c r="GF19" s="1"/>
-      <c r="GG19" s="1"/>
-      <c r="GH19" s="1"/>
-      <c r="GI19" s="1"/>
-      <c r="GJ19" s="1"/>
-      <c r="GK19" s="1"/>
-      <c r="GL19" s="1"/>
-      <c r="GM19" s="1"/>
-      <c r="GN19" s="1"/>
-      <c r="GO19" s="1"/>
-      <c r="GP19" s="1"/>
-      <c r="GQ19" s="1"/>
-      <c r="GR19" s="1"/>
-      <c r="GS19" s="1"/>
-      <c r="GT19" s="1"/>
-      <c r="GU19" s="1"/>
-      <c r="GV19" s="1"/>
-      <c r="GW19" s="1"/>
-      <c r="GX19" s="1"/>
-      <c r="GY19" s="1"/>
-      <c r="GZ19" s="1"/>
-      <c r="HA19" s="1"/>
-      <c r="HB19" s="1"/>
-      <c r="HC19" s="1"/>
-      <c r="HD19" s="1"/>
-      <c r="HE19" s="1"/>
-      <c r="HF19" s="1"/>
-      <c r="HG19" s="1"/>
-      <c r="HH19" s="1"/>
-      <c r="HI19" s="1"/>
-      <c r="HJ19" s="1"/>
-      <c r="HK19" s="1"/>
-      <c r="HL19" s="1"/>
-      <c r="HM19" s="1"/>
-      <c r="HN19" s="1"/>
-      <c r="HO19" s="1"/>
-      <c r="HP19" s="1"/>
-      <c r="HQ19" s="1"/>
-      <c r="HR19" s="1"/>
-      <c r="HS19" s="1"/>
-      <c r="HT19" s="1"/>
-      <c r="HU19" s="1"/>
-      <c r="HV19" s="1"/>
-      <c r="HW19" s="1"/>
-      <c r="HX19" s="1"/>
-      <c r="HY19" s="1"/>
-      <c r="HZ19" s="1"/>
-      <c r="IA19" s="1"/>
-      <c r="IB19" s="1"/>
-      <c r="IC19" s="1"/>
-      <c r="ID19" s="1"/>
-      <c r="IE19" s="1"/>
-      <c r="IF19" s="1"/>
-      <c r="IG19" s="1"/>
-      <c r="IH19" s="1"/>
-      <c r="II19" s="1"/>
-      <c r="IJ19" s="1"/>
-      <c r="IK19" s="1"/>
-      <c r="IL19" s="1"/>
-      <c r="IM19" s="1"/>
-      <c r="IN19" s="1"/>
-      <c r="IO19" s="1"/>
-      <c r="IP19" s="1"/>
-      <c r="IQ19" s="1"/>
-      <c r="IR19" s="1"/>
-      <c r="IS19" s="1"/>
-      <c r="IT19" s="1"/>
-      <c r="IU19" s="1"/>
-      <c r="IV19" s="1"/>
+      <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:256" ht="15.75" thickBot="1">
+    <row r="20" spans="1:256" ht="14.5">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
-      <c r="C20" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="98"/>
-      <c r="E20" s="98"/>
-      <c r="F20" s="98"/>
-      <c r="G20" s="98"/>
-      <c r="H20" s="29">
-        <f>H19+H18</f>
-        <v>60720.19</v>
-      </c>
+      <c r="C20" s="57" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="56"/>
+      <c r="E20" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="55"/>
+      <c r="G20" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="50"/>
       <c r="I20" s="4"/>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:256" ht="21.75" customHeight="1">
+    <row r="21" spans="1:256" ht="14.5">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
-      <c r="C21" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="26"/>
+      <c r="C21" s="57" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="56"/>
+      <c r="E21" s="55" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" s="55"/>
+      <c r="G21" s="58"/>
+      <c r="H21" s="50"/>
       <c r="I21" s="4"/>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:256" ht="15">
+    <row r="22" spans="1:256" ht="14.5">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
-      <c r="C22" s="72" t="s">
-        <v>26</v>
-      </c>
-      <c r="D22" s="73"/>
-      <c r="E22" s="73"/>
-      <c r="F22" s="73"/>
-      <c r="G22" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="H22" s="16"/>
+      <c r="C22" s="57" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22" s="56"/>
+      <c r="E22" s="55" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" s="55"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="50"/>
       <c r="I22" s="4"/>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:256" ht="15">
+    <row r="23" spans="1:256" ht="9.9" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
-      <c r="C23" s="66" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="67"/>
-      <c r="E23" s="68" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" s="68"/>
-      <c r="G23" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="H23" s="16"/>
+      <c r="C23" s="64"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="63"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="50"/>
       <c r="I23" s="4"/>
       <c r="J23" s="3"/>
     </row>
-    <row r="24" spans="1:256" ht="15">
+    <row r="24" spans="1:256" ht="14.5">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
-      <c r="C24" s="66" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24" s="67"/>
-      <c r="E24" s="68" t="s">
-        <v>22</v>
-      </c>
-      <c r="F24" s="68"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="16"/>
+      <c r="C24" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
+      <c r="G24" s="59" t="s">
+        <v>20</v>
+      </c>
+      <c r="H24" s="50"/>
       <c r="I24" s="4"/>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:256" ht="15">
+    <row r="25" spans="1:256" ht="14.5">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
-      <c r="C25" s="66" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25" s="67"/>
-      <c r="E25" s="68" t="s">
-        <v>22</v>
-      </c>
-      <c r="F25" s="68"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="16"/>
+      <c r="C25" s="57" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="56"/>
+      <c r="E25" s="55" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="55"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="50"/>
       <c r="I25" s="4"/>
       <c r="J25" s="3"/>
     </row>
-    <row r="26" spans="1:256" ht="9.9499999999999993" customHeight="1">
+    <row r="26" spans="1:256" ht="14.5">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="16"/>
+      <c r="C26" s="57" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="56"/>
+      <c r="E26" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="55"/>
+      <c r="G26" s="54">
+        <v>1</v>
+      </c>
+      <c r="H26" s="50"/>
       <c r="I26" s="4"/>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:256" ht="15">
+    <row r="27" spans="1:256" ht="14.5">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
-      <c r="C27" s="72" t="s">
-        <v>21</v>
-      </c>
-      <c r="D27" s="73"/>
-      <c r="E27" s="73"/>
-      <c r="F27" s="73"/>
-      <c r="G27" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="H27" s="16"/>
+      <c r="C27" s="57" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="56"/>
+      <c r="E27" s="55" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="55"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="50"/>
       <c r="I27" s="4"/>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:256" ht="15">
+    <row r="28" spans="1:256" ht="14.5">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
-      <c r="C28" s="66" t="s">
-        <v>17</v>
-      </c>
-      <c r="D28" s="67"/>
-      <c r="E28" s="68" t="s">
-        <v>19</v>
-      </c>
-      <c r="F28" s="68"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="16"/>
+      <c r="C28" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="56"/>
+      <c r="E28" s="55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" s="55"/>
+      <c r="G28" s="58"/>
+      <c r="H28" s="50"/>
       <c r="I28" s="4"/>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:256" ht="15">
+    <row r="29" spans="1:256" ht="14.5">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
-      <c r="C29" s="66" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="67"/>
-      <c r="E29" s="68" t="s">
-        <v>18</v>
-      </c>
-      <c r="F29" s="68"/>
-      <c r="G29" s="20">
-        <v>1</v>
-      </c>
-      <c r="H29" s="16"/>
+      <c r="C29" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="56"/>
+      <c r="E29" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="55"/>
+      <c r="G29" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="H29" s="50"/>
       <c r="I29" s="4"/>
       <c r="J29" s="3"/>
     </row>
-    <row r="30" spans="1:256" ht="15">
+    <row r="30" spans="1:256" ht="9.9" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
-      <c r="C30" s="66" t="s">
-        <v>17</v>
-      </c>
-      <c r="D30" s="67"/>
-      <c r="E30" s="68" t="s">
-        <v>16</v>
-      </c>
-      <c r="F30" s="68"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="16"/>
+      <c r="C30" s="53"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="52"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="50"/>
       <c r="I30" s="4"/>
       <c r="J30" s="3"/>
     </row>
-    <row r="31" spans="1:256" ht="15">
-      <c r="A31" s="3"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="66" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" s="67"/>
-      <c r="E31" s="68" t="s">
-        <v>14</v>
-      </c>
-      <c r="F31" s="68"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="3"/>
+    <row r="31" spans="1:256" s="5" customFormat="1" ht="14.5">
+      <c r="A31" s="6"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="48"/>
+      <c r="G31" s="48"/>
+      <c r="H31" s="47"/>
+      <c r="I31" s="46"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
+      <c r="W31" s="1"/>
+      <c r="X31" s="1"/>
+      <c r="Y31" s="1"/>
+      <c r="Z31" s="1"/>
+      <c r="AA31" s="1"/>
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="1"/>
+      <c r="AD31" s="1"/>
+      <c r="AE31" s="1"/>
+      <c r="AF31" s="1"/>
+      <c r="AG31" s="1"/>
+      <c r="AH31" s="1"/>
+      <c r="AI31" s="1"/>
+      <c r="AJ31" s="1"/>
+      <c r="AK31" s="1"/>
+      <c r="AL31" s="1"/>
+      <c r="AM31" s="1"/>
+      <c r="AN31" s="1"/>
+      <c r="AO31" s="1"/>
+      <c r="AP31" s="1"/>
+      <c r="AQ31" s="1"/>
+      <c r="AR31" s="1"/>
+      <c r="AS31" s="1"/>
+      <c r="AT31" s="1"/>
+      <c r="AU31" s="1"/>
+      <c r="AV31" s="1"/>
+      <c r="AW31" s="1"/>
+      <c r="AX31" s="1"/>
+      <c r="AY31" s="1"/>
+      <c r="AZ31" s="1"/>
+      <c r="BA31" s="1"/>
+      <c r="BB31" s="1"/>
+      <c r="BC31" s="1"/>
+      <c r="BD31" s="1"/>
+      <c r="BE31" s="1"/>
+      <c r="BF31" s="1"/>
+      <c r="BG31" s="1"/>
+      <c r="BH31" s="1"/>
+      <c r="BI31" s="1"/>
+      <c r="BJ31" s="1"/>
+      <c r="BK31" s="1"/>
+      <c r="BL31" s="1"/>
+      <c r="BM31" s="1"/>
+      <c r="BN31" s="1"/>
+      <c r="BO31" s="1"/>
+      <c r="BP31" s="1"/>
+      <c r="BQ31" s="1"/>
+      <c r="BR31" s="1"/>
+      <c r="BS31" s="1"/>
+      <c r="BT31" s="1"/>
+      <c r="BU31" s="1"/>
+      <c r="BV31" s="1"/>
+      <c r="BW31" s="1"/>
+      <c r="BX31" s="1"/>
+      <c r="BY31" s="1"/>
+      <c r="BZ31" s="1"/>
+      <c r="CA31" s="1"/>
+      <c r="CB31" s="1"/>
+      <c r="CC31" s="1"/>
+      <c r="CD31" s="1"/>
+      <c r="CE31" s="1"/>
+      <c r="CF31" s="1"/>
+      <c r="CG31" s="1"/>
+      <c r="CH31" s="1"/>
+      <c r="CI31" s="1"/>
+      <c r="CJ31" s="1"/>
+      <c r="CK31" s="1"/>
+      <c r="CL31" s="1"/>
+      <c r="CM31" s="1"/>
+      <c r="CN31" s="1"/>
+      <c r="CO31" s="1"/>
+      <c r="CP31" s="1"/>
+      <c r="CQ31" s="1"/>
+      <c r="CR31" s="1"/>
+      <c r="CS31" s="1"/>
+      <c r="CT31" s="1"/>
+      <c r="CU31" s="1"/>
+      <c r="CV31" s="1"/>
+      <c r="CW31" s="1"/>
+      <c r="CX31" s="1"/>
+      <c r="CY31" s="1"/>
+      <c r="CZ31" s="1"/>
+      <c r="DA31" s="1"/>
+      <c r="DB31" s="1"/>
+      <c r="DC31" s="1"/>
+      <c r="DD31" s="1"/>
+      <c r="DE31" s="1"/>
+      <c r="DF31" s="1"/>
+      <c r="DG31" s="1"/>
+      <c r="DH31" s="1"/>
+      <c r="DI31" s="1"/>
+      <c r="DJ31" s="1"/>
+      <c r="DK31" s="1"/>
+      <c r="DL31" s="1"/>
+      <c r="DM31" s="1"/>
+      <c r="DN31" s="1"/>
+      <c r="DO31" s="1"/>
+      <c r="DP31" s="1"/>
+      <c r="DQ31" s="1"/>
+      <c r="DR31" s="1"/>
+      <c r="DS31" s="1"/>
+      <c r="DT31" s="1"/>
+      <c r="DU31" s="1"/>
+      <c r="DV31" s="1"/>
+      <c r="DW31" s="1"/>
+      <c r="DX31" s="1"/>
+      <c r="DY31" s="1"/>
+      <c r="DZ31" s="1"/>
+      <c r="EA31" s="1"/>
+      <c r="EB31" s="1"/>
+      <c r="EC31" s="1"/>
+      <c r="ED31" s="1"/>
+      <c r="EE31" s="1"/>
+      <c r="EF31" s="1"/>
+      <c r="EG31" s="1"/>
+      <c r="EH31" s="1"/>
+      <c r="EI31" s="1"/>
+      <c r="EJ31" s="1"/>
+      <c r="EK31" s="1"/>
+      <c r="EL31" s="1"/>
+      <c r="EM31" s="1"/>
+      <c r="EN31" s="1"/>
+      <c r="EO31" s="1"/>
+      <c r="EP31" s="1"/>
+      <c r="EQ31" s="1"/>
+      <c r="ER31" s="1"/>
+      <c r="ES31" s="1"/>
+      <c r="ET31" s="1"/>
+      <c r="EU31" s="1"/>
+      <c r="EV31" s="1"/>
+      <c r="EW31" s="1"/>
+      <c r="EX31" s="1"/>
+      <c r="EY31" s="1"/>
+      <c r="EZ31" s="1"/>
+      <c r="FA31" s="1"/>
+      <c r="FB31" s="1"/>
+      <c r="FC31" s="1"/>
+      <c r="FD31" s="1"/>
+      <c r="FE31" s="1"/>
+      <c r="FF31" s="1"/>
+      <c r="FG31" s="1"/>
+      <c r="FH31" s="1"/>
+      <c r="FI31" s="1"/>
+      <c r="FJ31" s="1"/>
+      <c r="FK31" s="1"/>
+      <c r="FL31" s="1"/>
+      <c r="FM31" s="1"/>
+      <c r="FN31" s="1"/>
+      <c r="FO31" s="1"/>
+      <c r="FP31" s="1"/>
+      <c r="FQ31" s="1"/>
+      <c r="FR31" s="1"/>
+      <c r="FS31" s="1"/>
+      <c r="FT31" s="1"/>
+      <c r="FU31" s="1"/>
+      <c r="FV31" s="1"/>
+      <c r="FW31" s="1"/>
+      <c r="FX31" s="1"/>
+      <c r="FY31" s="1"/>
+      <c r="FZ31" s="1"/>
+      <c r="GA31" s="1"/>
+      <c r="GB31" s="1"/>
+      <c r="GC31" s="1"/>
+      <c r="GD31" s="1"/>
+      <c r="GE31" s="1"/>
+      <c r="GF31" s="1"/>
+      <c r="GG31" s="1"/>
+      <c r="GH31" s="1"/>
+      <c r="GI31" s="1"/>
+      <c r="GJ31" s="1"/>
+      <c r="GK31" s="1"/>
+      <c r="GL31" s="1"/>
+      <c r="GM31" s="1"/>
+      <c r="GN31" s="1"/>
+      <c r="GO31" s="1"/>
+      <c r="GP31" s="1"/>
+      <c r="GQ31" s="1"/>
+      <c r="GR31" s="1"/>
+      <c r="GS31" s="1"/>
+      <c r="GT31" s="1"/>
+      <c r="GU31" s="1"/>
+      <c r="GV31" s="1"/>
+      <c r="GW31" s="1"/>
+      <c r="GX31" s="1"/>
+      <c r="GY31" s="1"/>
+      <c r="GZ31" s="1"/>
+      <c r="HA31" s="1"/>
+      <c r="HB31" s="1"/>
+      <c r="HC31" s="1"/>
+      <c r="HD31" s="1"/>
+      <c r="HE31" s="1"/>
+      <c r="HF31" s="1"/>
+      <c r="HG31" s="1"/>
+      <c r="HH31" s="1"/>
+      <c r="HI31" s="1"/>
+      <c r="HJ31" s="1"/>
+      <c r="HK31" s="1"/>
+      <c r="HL31" s="1"/>
+      <c r="HM31" s="1"/>
+      <c r="HN31" s="1"/>
+      <c r="HO31" s="1"/>
+      <c r="HP31" s="1"/>
+      <c r="HQ31" s="1"/>
+      <c r="HR31" s="1"/>
+      <c r="HS31" s="1"/>
+      <c r="HT31" s="1"/>
+      <c r="HU31" s="1"/>
+      <c r="HV31" s="1"/>
+      <c r="HW31" s="1"/>
+      <c r="HX31" s="1"/>
+      <c r="HY31" s="1"/>
+      <c r="HZ31" s="1"/>
+      <c r="IA31" s="1"/>
+      <c r="IB31" s="1"/>
+      <c r="IC31" s="1"/>
+      <c r="ID31" s="1"/>
+      <c r="IE31" s="1"/>
+      <c r="IF31" s="1"/>
+      <c r="IG31" s="1"/>
+      <c r="IH31" s="1"/>
+      <c r="II31" s="1"/>
+      <c r="IJ31" s="1"/>
+      <c r="IK31" s="1"/>
+      <c r="IL31" s="1"/>
+      <c r="IM31" s="1"/>
+      <c r="IN31" s="1"/>
+      <c r="IO31" s="1"/>
+      <c r="IP31" s="1"/>
+      <c r="IQ31" s="1"/>
+      <c r="IR31" s="1"/>
+      <c r="IS31" s="1"/>
+      <c r="IT31" s="1"/>
+      <c r="IU31" s="1"/>
+      <c r="IV31" s="1"/>
     </row>
-    <row r="32" spans="1:256" ht="15">
-      <c r="A32" s="3"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="67"/>
-      <c r="E32" s="68" t="s">
-        <v>12</v>
-      </c>
-      <c r="F32" s="68"/>
-      <c r="G32" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="H32" s="16"/>
+    <row r="32" spans="1:256" s="5" customFormat="1" ht="39.9" customHeight="1">
+      <c r="A32" s="6"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="45" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="43"/>
       <c r="I32" s="4"/>
-      <c r="J32" s="3"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
+      <c r="T32" s="1"/>
+      <c r="U32" s="1"/>
+      <c r="V32" s="1"/>
+      <c r="W32" s="1"/>
+      <c r="X32" s="1"/>
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1"/>
+      <c r="AA32" s="1"/>
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="1"/>
+      <c r="AD32" s="1"/>
+      <c r="AE32" s="1"/>
+      <c r="AF32" s="1"/>
+      <c r="AG32" s="1"/>
+      <c r="AH32" s="1"/>
+      <c r="AI32" s="1"/>
+      <c r="AJ32" s="1"/>
+      <c r="AK32" s="1"/>
+      <c r="AL32" s="1"/>
+      <c r="AM32" s="1"/>
+      <c r="AN32" s="1"/>
+      <c r="AO32" s="1"/>
+      <c r="AP32" s="1"/>
+      <c r="AQ32" s="1"/>
+      <c r="AR32" s="1"/>
+      <c r="AS32" s="1"/>
+      <c r="AT32" s="1"/>
+      <c r="AU32" s="1"/>
+      <c r="AV32" s="1"/>
+      <c r="AW32" s="1"/>
+      <c r="AX32" s="1"/>
+      <c r="AY32" s="1"/>
+      <c r="AZ32" s="1"/>
+      <c r="BA32" s="1"/>
+      <c r="BB32" s="1"/>
+      <c r="BC32" s="1"/>
+      <c r="BD32" s="1"/>
+      <c r="BE32" s="1"/>
+      <c r="BF32" s="1"/>
+      <c r="BG32" s="1"/>
+      <c r="BH32" s="1"/>
+      <c r="BI32" s="1"/>
+      <c r="BJ32" s="1"/>
+      <c r="BK32" s="1"/>
+      <c r="BL32" s="1"/>
+      <c r="BM32" s="1"/>
+      <c r="BN32" s="1"/>
+      <c r="BO32" s="1"/>
+      <c r="BP32" s="1"/>
+      <c r="BQ32" s="1"/>
+      <c r="BR32" s="1"/>
+      <c r="BS32" s="1"/>
+      <c r="BT32" s="1"/>
+      <c r="BU32" s="1"/>
+      <c r="BV32" s="1"/>
+      <c r="BW32" s="1"/>
+      <c r="BX32" s="1"/>
+      <c r="BY32" s="1"/>
+      <c r="BZ32" s="1"/>
+      <c r="CA32" s="1"/>
+      <c r="CB32" s="1"/>
+      <c r="CC32" s="1"/>
+      <c r="CD32" s="1"/>
+      <c r="CE32" s="1"/>
+      <c r="CF32" s="1"/>
+      <c r="CG32" s="1"/>
+      <c r="CH32" s="1"/>
+      <c r="CI32" s="1"/>
+      <c r="CJ32" s="1"/>
+      <c r="CK32" s="1"/>
+      <c r="CL32" s="1"/>
+      <c r="CM32" s="1"/>
+      <c r="CN32" s="1"/>
+      <c r="CO32" s="1"/>
+      <c r="CP32" s="1"/>
+      <c r="CQ32" s="1"/>
+      <c r="CR32" s="1"/>
+      <c r="CS32" s="1"/>
+      <c r="CT32" s="1"/>
+      <c r="CU32" s="1"/>
+      <c r="CV32" s="1"/>
+      <c r="CW32" s="1"/>
+      <c r="CX32" s="1"/>
+      <c r="CY32" s="1"/>
+      <c r="CZ32" s="1"/>
+      <c r="DA32" s="1"/>
+      <c r="DB32" s="1"/>
+      <c r="DC32" s="1"/>
+      <c r="DD32" s="1"/>
+      <c r="DE32" s="1"/>
+      <c r="DF32" s="1"/>
+      <c r="DG32" s="1"/>
+      <c r="DH32" s="1"/>
+      <c r="DI32" s="1"/>
+      <c r="DJ32" s="1"/>
+      <c r="DK32" s="1"/>
+      <c r="DL32" s="1"/>
+      <c r="DM32" s="1"/>
+      <c r="DN32" s="1"/>
+      <c r="DO32" s="1"/>
+      <c r="DP32" s="1"/>
+      <c r="DQ32" s="1"/>
+      <c r="DR32" s="1"/>
+      <c r="DS32" s="1"/>
+      <c r="DT32" s="1"/>
+      <c r="DU32" s="1"/>
+      <c r="DV32" s="1"/>
+      <c r="DW32" s="1"/>
+      <c r="DX32" s="1"/>
+      <c r="DY32" s="1"/>
+      <c r="DZ32" s="1"/>
+      <c r="EA32" s="1"/>
+      <c r="EB32" s="1"/>
+      <c r="EC32" s="1"/>
+      <c r="ED32" s="1"/>
+      <c r="EE32" s="1"/>
+      <c r="EF32" s="1"/>
+      <c r="EG32" s="1"/>
+      <c r="EH32" s="1"/>
+      <c r="EI32" s="1"/>
+      <c r="EJ32" s="1"/>
+      <c r="EK32" s="1"/>
+      <c r="EL32" s="1"/>
+      <c r="EM32" s="1"/>
+      <c r="EN32" s="1"/>
+      <c r="EO32" s="1"/>
+      <c r="EP32" s="1"/>
+      <c r="EQ32" s="1"/>
+      <c r="ER32" s="1"/>
+      <c r="ES32" s="1"/>
+      <c r="ET32" s="1"/>
+      <c r="EU32" s="1"/>
+      <c r="EV32" s="1"/>
+      <c r="EW32" s="1"/>
+      <c r="EX32" s="1"/>
+      <c r="EY32" s="1"/>
+      <c r="EZ32" s="1"/>
+      <c r="FA32" s="1"/>
+      <c r="FB32" s="1"/>
+      <c r="FC32" s="1"/>
+      <c r="FD32" s="1"/>
+      <c r="FE32" s="1"/>
+      <c r="FF32" s="1"/>
+      <c r="FG32" s="1"/>
+      <c r="FH32" s="1"/>
+      <c r="FI32" s="1"/>
+      <c r="FJ32" s="1"/>
+      <c r="FK32" s="1"/>
+      <c r="FL32" s="1"/>
+      <c r="FM32" s="1"/>
+      <c r="FN32" s="1"/>
+      <c r="FO32" s="1"/>
+      <c r="FP32" s="1"/>
+      <c r="FQ32" s="1"/>
+      <c r="FR32" s="1"/>
+      <c r="FS32" s="1"/>
+      <c r="FT32" s="1"/>
+      <c r="FU32" s="1"/>
+      <c r="FV32" s="1"/>
+      <c r="FW32" s="1"/>
+      <c r="FX32" s="1"/>
+      <c r="FY32" s="1"/>
+      <c r="FZ32" s="1"/>
+      <c r="GA32" s="1"/>
+      <c r="GB32" s="1"/>
+      <c r="GC32" s="1"/>
+      <c r="GD32" s="1"/>
+      <c r="GE32" s="1"/>
+      <c r="GF32" s="1"/>
+      <c r="GG32" s="1"/>
+      <c r="GH32" s="1"/>
+      <c r="GI32" s="1"/>
+      <c r="GJ32" s="1"/>
+      <c r="GK32" s="1"/>
+      <c r="GL32" s="1"/>
+      <c r="GM32" s="1"/>
+      <c r="GN32" s="1"/>
+      <c r="GO32" s="1"/>
+      <c r="GP32" s="1"/>
+      <c r="GQ32" s="1"/>
+      <c r="GR32" s="1"/>
+      <c r="GS32" s="1"/>
+      <c r="GT32" s="1"/>
+      <c r="GU32" s="1"/>
+      <c r="GV32" s="1"/>
+      <c r="GW32" s="1"/>
+      <c r="GX32" s="1"/>
+      <c r="GY32" s="1"/>
+      <c r="GZ32" s="1"/>
+      <c r="HA32" s="1"/>
+      <c r="HB32" s="1"/>
+      <c r="HC32" s="1"/>
+      <c r="HD32" s="1"/>
+      <c r="HE32" s="1"/>
+      <c r="HF32" s="1"/>
+      <c r="HG32" s="1"/>
+      <c r="HH32" s="1"/>
+      <c r="HI32" s="1"/>
+      <c r="HJ32" s="1"/>
+      <c r="HK32" s="1"/>
+      <c r="HL32" s="1"/>
+      <c r="HM32" s="1"/>
+      <c r="HN32" s="1"/>
+      <c r="HO32" s="1"/>
+      <c r="HP32" s="1"/>
+      <c r="HQ32" s="1"/>
+      <c r="HR32" s="1"/>
+      <c r="HS32" s="1"/>
+      <c r="HT32" s="1"/>
+      <c r="HU32" s="1"/>
+      <c r="HV32" s="1"/>
+      <c r="HW32" s="1"/>
+      <c r="HX32" s="1"/>
+      <c r="HY32" s="1"/>
+      <c r="HZ32" s="1"/>
+      <c r="IA32" s="1"/>
+      <c r="IB32" s="1"/>
+      <c r="IC32" s="1"/>
+      <c r="ID32" s="1"/>
+      <c r="IE32" s="1"/>
+      <c r="IF32" s="1"/>
+      <c r="IG32" s="1"/>
+      <c r="IH32" s="1"/>
+      <c r="II32" s="1"/>
+      <c r="IJ32" s="1"/>
+      <c r="IK32" s="1"/>
+      <c r="IL32" s="1"/>
+      <c r="IM32" s="1"/>
+      <c r="IN32" s="1"/>
+      <c r="IO32" s="1"/>
+      <c r="IP32" s="1"/>
+      <c r="IQ32" s="1"/>
+      <c r="IR32" s="1"/>
+      <c r="IS32" s="1"/>
+      <c r="IT32" s="1"/>
+      <c r="IU32" s="1"/>
+      <c r="IV32" s="1"/>
     </row>
-    <row r="33" spans="1:256" ht="9.9499999999999993" customHeight="1">
-      <c r="A33" s="3"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="16"/>
+    <row r="33" spans="1:256" s="5" customFormat="1" ht="39.9" customHeight="1">
+      <c r="A33" s="6"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="40"/>
       <c r="I33" s="4"/>
-      <c r="J33" s="3"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
+      <c r="T33" s="1"/>
+      <c r="U33" s="1"/>
+      <c r="V33" s="1"/>
+      <c r="W33" s="1"/>
+      <c r="X33" s="1"/>
+      <c r="Y33" s="1"/>
+      <c r="Z33" s="1"/>
+      <c r="AA33" s="1"/>
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1"/>
+      <c r="AD33" s="1"/>
+      <c r="AE33" s="1"/>
+      <c r="AF33" s="1"/>
+      <c r="AG33" s="1"/>
+      <c r="AH33" s="1"/>
+      <c r="AI33" s="1"/>
+      <c r="AJ33" s="1"/>
+      <c r="AK33" s="1"/>
+      <c r="AL33" s="1"/>
+      <c r="AM33" s="1"/>
+      <c r="AN33" s="1"/>
+      <c r="AO33" s="1"/>
+      <c r="AP33" s="1"/>
+      <c r="AQ33" s="1"/>
+      <c r="AR33" s="1"/>
+      <c r="AS33" s="1"/>
+      <c r="AT33" s="1"/>
+      <c r="AU33" s="1"/>
+      <c r="AV33" s="1"/>
+      <c r="AW33" s="1"/>
+      <c r="AX33" s="1"/>
+      <c r="AY33" s="1"/>
+      <c r="AZ33" s="1"/>
+      <c r="BA33" s="1"/>
+      <c r="BB33" s="1"/>
+      <c r="BC33" s="1"/>
+      <c r="BD33" s="1"/>
+      <c r="BE33" s="1"/>
+      <c r="BF33" s="1"/>
+      <c r="BG33" s="1"/>
+      <c r="BH33" s="1"/>
+      <c r="BI33" s="1"/>
+      <c r="BJ33" s="1"/>
+      <c r="BK33" s="1"/>
+      <c r="BL33" s="1"/>
+      <c r="BM33" s="1"/>
+      <c r="BN33" s="1"/>
+      <c r="BO33" s="1"/>
+      <c r="BP33" s="1"/>
+      <c r="BQ33" s="1"/>
+      <c r="BR33" s="1"/>
+      <c r="BS33" s="1"/>
+      <c r="BT33" s="1"/>
+      <c r="BU33" s="1"/>
+      <c r="BV33" s="1"/>
+      <c r="BW33" s="1"/>
+      <c r="BX33" s="1"/>
+      <c r="BY33" s="1"/>
+      <c r="BZ33" s="1"/>
+      <c r="CA33" s="1"/>
+      <c r="CB33" s="1"/>
+      <c r="CC33" s="1"/>
+      <c r="CD33" s="1"/>
+      <c r="CE33" s="1"/>
+      <c r="CF33" s="1"/>
+      <c r="CG33" s="1"/>
+      <c r="CH33" s="1"/>
+      <c r="CI33" s="1"/>
+      <c r="CJ33" s="1"/>
+      <c r="CK33" s="1"/>
+      <c r="CL33" s="1"/>
+      <c r="CM33" s="1"/>
+      <c r="CN33" s="1"/>
+      <c r="CO33" s="1"/>
+      <c r="CP33" s="1"/>
+      <c r="CQ33" s="1"/>
+      <c r="CR33" s="1"/>
+      <c r="CS33" s="1"/>
+      <c r="CT33" s="1"/>
+      <c r="CU33" s="1"/>
+      <c r="CV33" s="1"/>
+      <c r="CW33" s="1"/>
+      <c r="CX33" s="1"/>
+      <c r="CY33" s="1"/>
+      <c r="CZ33" s="1"/>
+      <c r="DA33" s="1"/>
+      <c r="DB33" s="1"/>
+      <c r="DC33" s="1"/>
+      <c r="DD33" s="1"/>
+      <c r="DE33" s="1"/>
+      <c r="DF33" s="1"/>
+      <c r="DG33" s="1"/>
+      <c r="DH33" s="1"/>
+      <c r="DI33" s="1"/>
+      <c r="DJ33" s="1"/>
+      <c r="DK33" s="1"/>
+      <c r="DL33" s="1"/>
+      <c r="DM33" s="1"/>
+      <c r="DN33" s="1"/>
+      <c r="DO33" s="1"/>
+      <c r="DP33" s="1"/>
+      <c r="DQ33" s="1"/>
+      <c r="DR33" s="1"/>
+      <c r="DS33" s="1"/>
+      <c r="DT33" s="1"/>
+      <c r="DU33" s="1"/>
+      <c r="DV33" s="1"/>
+      <c r="DW33" s="1"/>
+      <c r="DX33" s="1"/>
+      <c r="DY33" s="1"/>
+      <c r="DZ33" s="1"/>
+      <c r="EA33" s="1"/>
+      <c r="EB33" s="1"/>
+      <c r="EC33" s="1"/>
+      <c r="ED33" s="1"/>
+      <c r="EE33" s="1"/>
+      <c r="EF33" s="1"/>
+      <c r="EG33" s="1"/>
+      <c r="EH33" s="1"/>
+      <c r="EI33" s="1"/>
+      <c r="EJ33" s="1"/>
+      <c r="EK33" s="1"/>
+      <c r="EL33" s="1"/>
+      <c r="EM33" s="1"/>
+      <c r="EN33" s="1"/>
+      <c r="EO33" s="1"/>
+      <c r="EP33" s="1"/>
+      <c r="EQ33" s="1"/>
+      <c r="ER33" s="1"/>
+      <c r="ES33" s="1"/>
+      <c r="ET33" s="1"/>
+      <c r="EU33" s="1"/>
+      <c r="EV33" s="1"/>
+      <c r="EW33" s="1"/>
+      <c r="EX33" s="1"/>
+      <c r="EY33" s="1"/>
+      <c r="EZ33" s="1"/>
+      <c r="FA33" s="1"/>
+      <c r="FB33" s="1"/>
+      <c r="FC33" s="1"/>
+      <c r="FD33" s="1"/>
+      <c r="FE33" s="1"/>
+      <c r="FF33" s="1"/>
+      <c r="FG33" s="1"/>
+      <c r="FH33" s="1"/>
+      <c r="FI33" s="1"/>
+      <c r="FJ33" s="1"/>
+      <c r="FK33" s="1"/>
+      <c r="FL33" s="1"/>
+      <c r="FM33" s="1"/>
+      <c r="FN33" s="1"/>
+      <c r="FO33" s="1"/>
+      <c r="FP33" s="1"/>
+      <c r="FQ33" s="1"/>
+      <c r="FR33" s="1"/>
+      <c r="FS33" s="1"/>
+      <c r="FT33" s="1"/>
+      <c r="FU33" s="1"/>
+      <c r="FV33" s="1"/>
+      <c r="FW33" s="1"/>
+      <c r="FX33" s="1"/>
+      <c r="FY33" s="1"/>
+      <c r="FZ33" s="1"/>
+      <c r="GA33" s="1"/>
+      <c r="GB33" s="1"/>
+      <c r="GC33" s="1"/>
+      <c r="GD33" s="1"/>
+      <c r="GE33" s="1"/>
+      <c r="GF33" s="1"/>
+      <c r="GG33" s="1"/>
+      <c r="GH33" s="1"/>
+      <c r="GI33" s="1"/>
+      <c r="GJ33" s="1"/>
+      <c r="GK33" s="1"/>
+      <c r="GL33" s="1"/>
+      <c r="GM33" s="1"/>
+      <c r="GN33" s="1"/>
+      <c r="GO33" s="1"/>
+      <c r="GP33" s="1"/>
+      <c r="GQ33" s="1"/>
+      <c r="GR33" s="1"/>
+      <c r="GS33" s="1"/>
+      <c r="GT33" s="1"/>
+      <c r="GU33" s="1"/>
+      <c r="GV33" s="1"/>
+      <c r="GW33" s="1"/>
+      <c r="GX33" s="1"/>
+      <c r="GY33" s="1"/>
+      <c r="GZ33" s="1"/>
+      <c r="HA33" s="1"/>
+      <c r="HB33" s="1"/>
+      <c r="HC33" s="1"/>
+      <c r="HD33" s="1"/>
+      <c r="HE33" s="1"/>
+      <c r="HF33" s="1"/>
+      <c r="HG33" s="1"/>
+      <c r="HH33" s="1"/>
+      <c r="HI33" s="1"/>
+      <c r="HJ33" s="1"/>
+      <c r="HK33" s="1"/>
+      <c r="HL33" s="1"/>
+      <c r="HM33" s="1"/>
+      <c r="HN33" s="1"/>
+      <c r="HO33" s="1"/>
+      <c r="HP33" s="1"/>
+      <c r="HQ33" s="1"/>
+      <c r="HR33" s="1"/>
+      <c r="HS33" s="1"/>
+      <c r="HT33" s="1"/>
+      <c r="HU33" s="1"/>
+      <c r="HV33" s="1"/>
+      <c r="HW33" s="1"/>
+      <c r="HX33" s="1"/>
+      <c r="HY33" s="1"/>
+      <c r="HZ33" s="1"/>
+      <c r="IA33" s="1"/>
+      <c r="IB33" s="1"/>
+      <c r="IC33" s="1"/>
+      <c r="ID33" s="1"/>
+      <c r="IE33" s="1"/>
+      <c r="IF33" s="1"/>
+      <c r="IG33" s="1"/>
+      <c r="IH33" s="1"/>
+      <c r="II33" s="1"/>
+      <c r="IJ33" s="1"/>
+      <c r="IK33" s="1"/>
+      <c r="IL33" s="1"/>
+      <c r="IM33" s="1"/>
+      <c r="IN33" s="1"/>
+      <c r="IO33" s="1"/>
+      <c r="IP33" s="1"/>
+      <c r="IQ33" s="1"/>
+      <c r="IR33" s="1"/>
+      <c r="IS33" s="1"/>
+      <c r="IT33" s="1"/>
+      <c r="IU33" s="1"/>
+      <c r="IV33" s="1"/>
     </row>
-    <row r="34" spans="1:256" s="5" customFormat="1" ht="15">
+    <row r="34" spans="1:256" s="5" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
       <c r="A34" s="6"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="69" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" s="70"/>
-      <c r="E34" s="70"/>
-      <c r="F34" s="70"/>
-      <c r="G34" s="70"/>
-      <c r="H34" s="71"/>
-      <c r="I34" s="15"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="37"/>
+      <c r="I34" s="4"/>
       <c r="J34" s="6"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
@@ -3170,17 +3907,17 @@
       <c r="IU34" s="1"/>
       <c r="IV34" s="1"/>
     </row>
-    <row r="35" spans="1:256" s="5" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="35" spans="1:256" s="5" customFormat="1" ht="14.5">
       <c r="A35" s="6"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="77" t="s">
-        <v>9</v>
-      </c>
-      <c r="D35" s="78"/>
-      <c r="E35" s="78"/>
-      <c r="F35" s="78"/>
-      <c r="G35" s="78"/>
-      <c r="H35" s="79"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="35"/>
+      <c r="E35" s="35"/>
+      <c r="F35" s="35"/>
+      <c r="G35" s="35"/>
+      <c r="H35" s="34"/>
       <c r="I35" s="4"/>
       <c r="J35" s="6"/>
       <c r="K35" s="1"/>
@@ -3430,15 +4167,21 @@
       <c r="IU35" s="1"/>
       <c r="IV35" s="1"/>
     </row>
-    <row r="36" spans="1:256" s="5" customFormat="1" ht="39.950000000000003" customHeight="1">
+    <row r="36" spans="1:256" s="5" customFormat="1" ht="14.5">
       <c r="A36" s="6"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="80"/>
-      <c r="D36" s="81"/>
-      <c r="E36" s="81"/>
-      <c r="F36" s="81"/>
-      <c r="G36" s="81"/>
-      <c r="H36" s="82"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="32"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="G36" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="H36" s="28"/>
       <c r="I36" s="4"/>
       <c r="J36" s="6"/>
       <c r="K36" s="1"/>
@@ -3688,15 +4431,17 @@
       <c r="IU36" s="1"/>
       <c r="IV36" s="1"/>
     </row>
-    <row r="37" spans="1:256" s="5" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1">
+    <row r="37" spans="1:256" s="5" customFormat="1" ht="21">
       <c r="A37" s="6"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="83"/>
-      <c r="D37" s="84"/>
-      <c r="E37" s="84"/>
-      <c r="F37" s="84"/>
-      <c r="G37" s="84"/>
-      <c r="H37" s="85"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" s="24"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="23"/>
       <c r="I37" s="4"/>
       <c r="J37" s="6"/>
       <c r="K37" s="1"/>
@@ -3946,17 +4691,22 @@
       <c r="IU37" s="1"/>
       <c r="IV37" s="1"/>
     </row>
-    <row r="38" spans="1:256" s="5" customFormat="1" ht="15">
+    <row r="38" spans="1:256" s="5" customFormat="1" ht="21.5">
       <c r="A38" s="6"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="86" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="87"/>
-      <c r="E38" s="87"/>
-      <c r="F38" s="87"/>
-      <c r="G38" s="87"/>
-      <c r="H38" s="88"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="22" t="str">
+        <f>E29</f>
+        <v>Favio Melo</v>
+      </c>
+      <c r="D38" s="21"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="H38" s="17"/>
       <c r="I38" s="4"/>
       <c r="J38" s="6"/>
       <c r="K38" s="1"/>
@@ -4206,21 +4956,15 @@
       <c r="IU38" s="1"/>
       <c r="IV38" s="1"/>
     </row>
-    <row r="39" spans="1:256" s="5" customFormat="1" ht="15">
+    <row r="39" spans="1:256" s="5" customFormat="1" ht="9.9" customHeight="1">
       <c r="A39" s="6"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="74" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" s="75"/>
-      <c r="E39" s="76"/>
-      <c r="F39" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="G39" s="64" t="s">
-        <v>5</v>
-      </c>
-      <c r="H39" s="65"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="14"/>
       <c r="I39" s="4"/>
       <c r="J39" s="6"/>
       <c r="K39" s="1"/>
@@ -4470,17 +5214,17 @@
       <c r="IU39" s="1"/>
       <c r="IV39" s="1"/>
     </row>
-    <row r="40" spans="1:256" s="5" customFormat="1" ht="21">
+    <row r="40" spans="1:256" s="5" customFormat="1" ht="21" customHeight="1">
       <c r="A40" s="6"/>
-      <c r="B40" s="7"/>
+      <c r="B40" s="10"/>
       <c r="C40" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D40" s="10"/>
+        <v>1</v>
+      </c>
+      <c r="D40" s="12"/>
       <c r="E40" s="12"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="9"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="11"/>
       <c r="I40" s="4"/>
       <c r="J40" s="6"/>
       <c r="K40" s="1"/>
@@ -4730,22 +5474,17 @@
       <c r="IU40" s="1"/>
       <c r="IV40" s="1"/>
     </row>
-    <row r="41" spans="1:256" s="5" customFormat="1" ht="21">
+    <row r="41" spans="1:256" s="5" customFormat="1" ht="21" customHeight="1" thickBot="1">
       <c r="A41" s="6"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="50" t="str">
-        <f>E32</f>
-        <v>Favio Melo</v>
-      </c>
-      <c r="D41" s="51"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="G41" s="53" t="s">
-        <v>2</v>
-      </c>
-      <c r="H41" s="54"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8"/>
+      <c r="H41" s="7"/>
       <c r="I41" s="4"/>
       <c r="J41" s="6"/>
       <c r="K41" s="1"/>
@@ -4995,856 +5734,78 @@
       <c r="IU41" s="1"/>
       <c r="IV41" s="1"/>
     </row>
-    <row r="42" spans="1:256" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1">
-      <c r="A42" s="6"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="56"/>
-      <c r="E42" s="56"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="56"/>
-      <c r="H42" s="57"/>
+    <row r="42" spans="1:256" ht="14">
+      <c r="A42" s="3"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
       <c r="I42" s="4"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="1"/>
-      <c r="L42" s="1"/>
-      <c r="M42" s="1"/>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1"/>
-      <c r="P42" s="1"/>
-      <c r="Q42" s="1"/>
-      <c r="R42" s="1"/>
-      <c r="S42" s="1"/>
-      <c r="T42" s="1"/>
-      <c r="U42" s="1"/>
-      <c r="V42" s="1"/>
-      <c r="W42" s="1"/>
-      <c r="X42" s="1"/>
-      <c r="Y42" s="1"/>
-      <c r="Z42" s="1"/>
-      <c r="AA42" s="1"/>
-      <c r="AB42" s="1"/>
-      <c r="AC42" s="1"/>
-      <c r="AD42" s="1"/>
-      <c r="AE42" s="1"/>
-      <c r="AF42" s="1"/>
-      <c r="AG42" s="1"/>
-      <c r="AH42" s="1"/>
-      <c r="AI42" s="1"/>
-      <c r="AJ42" s="1"/>
-      <c r="AK42" s="1"/>
-      <c r="AL42" s="1"/>
-      <c r="AM42" s="1"/>
-      <c r="AN42" s="1"/>
-      <c r="AO42" s="1"/>
-      <c r="AP42" s="1"/>
-      <c r="AQ42" s="1"/>
-      <c r="AR42" s="1"/>
-      <c r="AS42" s="1"/>
-      <c r="AT42" s="1"/>
-      <c r="AU42" s="1"/>
-      <c r="AV42" s="1"/>
-      <c r="AW42" s="1"/>
-      <c r="AX42" s="1"/>
-      <c r="AY42" s="1"/>
-      <c r="AZ42" s="1"/>
-      <c r="BA42" s="1"/>
-      <c r="BB42" s="1"/>
-      <c r="BC42" s="1"/>
-      <c r="BD42" s="1"/>
-      <c r="BE42" s="1"/>
-      <c r="BF42" s="1"/>
-      <c r="BG42" s="1"/>
-      <c r="BH42" s="1"/>
-      <c r="BI42" s="1"/>
-      <c r="BJ42" s="1"/>
-      <c r="BK42" s="1"/>
-      <c r="BL42" s="1"/>
-      <c r="BM42" s="1"/>
-      <c r="BN42" s="1"/>
-      <c r="BO42" s="1"/>
-      <c r="BP42" s="1"/>
-      <c r="BQ42" s="1"/>
-      <c r="BR42" s="1"/>
-      <c r="BS42" s="1"/>
-      <c r="BT42" s="1"/>
-      <c r="BU42" s="1"/>
-      <c r="BV42" s="1"/>
-      <c r="BW42" s="1"/>
-      <c r="BX42" s="1"/>
-      <c r="BY42" s="1"/>
-      <c r="BZ42" s="1"/>
-      <c r="CA42" s="1"/>
-      <c r="CB42" s="1"/>
-      <c r="CC42" s="1"/>
-      <c r="CD42" s="1"/>
-      <c r="CE42" s="1"/>
-      <c r="CF42" s="1"/>
-      <c r="CG42" s="1"/>
-      <c r="CH42" s="1"/>
-      <c r="CI42" s="1"/>
-      <c r="CJ42" s="1"/>
-      <c r="CK42" s="1"/>
-      <c r="CL42" s="1"/>
-      <c r="CM42" s="1"/>
-      <c r="CN42" s="1"/>
-      <c r="CO42" s="1"/>
-      <c r="CP42" s="1"/>
-      <c r="CQ42" s="1"/>
-      <c r="CR42" s="1"/>
-      <c r="CS42" s="1"/>
-      <c r="CT42" s="1"/>
-      <c r="CU42" s="1"/>
-      <c r="CV42" s="1"/>
-      <c r="CW42" s="1"/>
-      <c r="CX42" s="1"/>
-      <c r="CY42" s="1"/>
-      <c r="CZ42" s="1"/>
-      <c r="DA42" s="1"/>
-      <c r="DB42" s="1"/>
-      <c r="DC42" s="1"/>
-      <c r="DD42" s="1"/>
-      <c r="DE42" s="1"/>
-      <c r="DF42" s="1"/>
-      <c r="DG42" s="1"/>
-      <c r="DH42" s="1"/>
-      <c r="DI42" s="1"/>
-      <c r="DJ42" s="1"/>
-      <c r="DK42" s="1"/>
-      <c r="DL42" s="1"/>
-      <c r="DM42" s="1"/>
-      <c r="DN42" s="1"/>
-      <c r="DO42" s="1"/>
-      <c r="DP42" s="1"/>
-      <c r="DQ42" s="1"/>
-      <c r="DR42" s="1"/>
-      <c r="DS42" s="1"/>
-      <c r="DT42" s="1"/>
-      <c r="DU42" s="1"/>
-      <c r="DV42" s="1"/>
-      <c r="DW42" s="1"/>
-      <c r="DX42" s="1"/>
-      <c r="DY42" s="1"/>
-      <c r="DZ42" s="1"/>
-      <c r="EA42" s="1"/>
-      <c r="EB42" s="1"/>
-      <c r="EC42" s="1"/>
-      <c r="ED42" s="1"/>
-      <c r="EE42" s="1"/>
-      <c r="EF42" s="1"/>
-      <c r="EG42" s="1"/>
-      <c r="EH42" s="1"/>
-      <c r="EI42" s="1"/>
-      <c r="EJ42" s="1"/>
-      <c r="EK42" s="1"/>
-      <c r="EL42" s="1"/>
-      <c r="EM42" s="1"/>
-      <c r="EN42" s="1"/>
-      <c r="EO42" s="1"/>
-      <c r="EP42" s="1"/>
-      <c r="EQ42" s="1"/>
-      <c r="ER42" s="1"/>
-      <c r="ES42" s="1"/>
-      <c r="ET42" s="1"/>
-      <c r="EU42" s="1"/>
-      <c r="EV42" s="1"/>
-      <c r="EW42" s="1"/>
-      <c r="EX42" s="1"/>
-      <c r="EY42" s="1"/>
-      <c r="EZ42" s="1"/>
-      <c r="FA42" s="1"/>
-      <c r="FB42" s="1"/>
-      <c r="FC42" s="1"/>
-      <c r="FD42" s="1"/>
-      <c r="FE42" s="1"/>
-      <c r="FF42" s="1"/>
-      <c r="FG42" s="1"/>
-      <c r="FH42" s="1"/>
-      <c r="FI42" s="1"/>
-      <c r="FJ42" s="1"/>
-      <c r="FK42" s="1"/>
-      <c r="FL42" s="1"/>
-      <c r="FM42" s="1"/>
-      <c r="FN42" s="1"/>
-      <c r="FO42" s="1"/>
-      <c r="FP42" s="1"/>
-      <c r="FQ42" s="1"/>
-      <c r="FR42" s="1"/>
-      <c r="FS42" s="1"/>
-      <c r="FT42" s="1"/>
-      <c r="FU42" s="1"/>
-      <c r="FV42" s="1"/>
-      <c r="FW42" s="1"/>
-      <c r="FX42" s="1"/>
-      <c r="FY42" s="1"/>
-      <c r="FZ42" s="1"/>
-      <c r="GA42" s="1"/>
-      <c r="GB42" s="1"/>
-      <c r="GC42" s="1"/>
-      <c r="GD42" s="1"/>
-      <c r="GE42" s="1"/>
-      <c r="GF42" s="1"/>
-      <c r="GG42" s="1"/>
-      <c r="GH42" s="1"/>
-      <c r="GI42" s="1"/>
-      <c r="GJ42" s="1"/>
-      <c r="GK42" s="1"/>
-      <c r="GL42" s="1"/>
-      <c r="GM42" s="1"/>
-      <c r="GN42" s="1"/>
-      <c r="GO42" s="1"/>
-      <c r="GP42" s="1"/>
-      <c r="GQ42" s="1"/>
-      <c r="GR42" s="1"/>
-      <c r="GS42" s="1"/>
-      <c r="GT42" s="1"/>
-      <c r="GU42" s="1"/>
-      <c r="GV42" s="1"/>
-      <c r="GW42" s="1"/>
-      <c r="GX42" s="1"/>
-      <c r="GY42" s="1"/>
-      <c r="GZ42" s="1"/>
-      <c r="HA42" s="1"/>
-      <c r="HB42" s="1"/>
-      <c r="HC42" s="1"/>
-      <c r="HD42" s="1"/>
-      <c r="HE42" s="1"/>
-      <c r="HF42" s="1"/>
-      <c r="HG42" s="1"/>
-      <c r="HH42" s="1"/>
-      <c r="HI42" s="1"/>
-      <c r="HJ42" s="1"/>
-      <c r="HK42" s="1"/>
-      <c r="HL42" s="1"/>
-      <c r="HM42" s="1"/>
-      <c r="HN42" s="1"/>
-      <c r="HO42" s="1"/>
-      <c r="HP42" s="1"/>
-      <c r="HQ42" s="1"/>
-      <c r="HR42" s="1"/>
-      <c r="HS42" s="1"/>
-      <c r="HT42" s="1"/>
-      <c r="HU42" s="1"/>
-      <c r="HV42" s="1"/>
-      <c r="HW42" s="1"/>
-      <c r="HX42" s="1"/>
-      <c r="HY42" s="1"/>
-      <c r="HZ42" s="1"/>
-      <c r="IA42" s="1"/>
-      <c r="IB42" s="1"/>
-      <c r="IC42" s="1"/>
-      <c r="ID42" s="1"/>
-      <c r="IE42" s="1"/>
-      <c r="IF42" s="1"/>
-      <c r="IG42" s="1"/>
-      <c r="IH42" s="1"/>
-      <c r="II42" s="1"/>
-      <c r="IJ42" s="1"/>
-      <c r="IK42" s="1"/>
-      <c r="IL42" s="1"/>
-      <c r="IM42" s="1"/>
-      <c r="IN42" s="1"/>
-      <c r="IO42" s="1"/>
-      <c r="IP42" s="1"/>
-      <c r="IQ42" s="1"/>
-      <c r="IR42" s="1"/>
-      <c r="IS42" s="1"/>
-      <c r="IT42" s="1"/>
-      <c r="IU42" s="1"/>
-      <c r="IV42" s="1"/>
+      <c r="J42" s="3"/>
     </row>
-    <row r="43" spans="1:256" s="5" customFormat="1" ht="21" customHeight="1">
-      <c r="A43" s="6"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="58" t="s">
-        <v>1</v>
-      </c>
-      <c r="D43" s="59"/>
-      <c r="E43" s="59"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
-      <c r="H43" s="60"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="6"/>
-      <c r="K43" s="1"/>
-      <c r="L43" s="1"/>
-      <c r="M43" s="1"/>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
-      <c r="P43" s="1"/>
-      <c r="Q43" s="1"/>
-      <c r="R43" s="1"/>
-      <c r="S43" s="1"/>
-      <c r="T43" s="1"/>
-      <c r="U43" s="1"/>
-      <c r="V43" s="1"/>
-      <c r="W43" s="1"/>
-      <c r="X43" s="1"/>
-      <c r="Y43" s="1"/>
-      <c r="Z43" s="1"/>
-      <c r="AA43" s="1"/>
-      <c r="AB43" s="1"/>
-      <c r="AC43" s="1"/>
-      <c r="AD43" s="1"/>
-      <c r="AE43" s="1"/>
-      <c r="AF43" s="1"/>
-      <c r="AG43" s="1"/>
-      <c r="AH43" s="1"/>
-      <c r="AI43" s="1"/>
-      <c r="AJ43" s="1"/>
-      <c r="AK43" s="1"/>
-      <c r="AL43" s="1"/>
-      <c r="AM43" s="1"/>
-      <c r="AN43" s="1"/>
-      <c r="AO43" s="1"/>
-      <c r="AP43" s="1"/>
-      <c r="AQ43" s="1"/>
-      <c r="AR43" s="1"/>
-      <c r="AS43" s="1"/>
-      <c r="AT43" s="1"/>
-      <c r="AU43" s="1"/>
-      <c r="AV43" s="1"/>
-      <c r="AW43" s="1"/>
-      <c r="AX43" s="1"/>
-      <c r="AY43" s="1"/>
-      <c r="AZ43" s="1"/>
-      <c r="BA43" s="1"/>
-      <c r="BB43" s="1"/>
-      <c r="BC43" s="1"/>
-      <c r="BD43" s="1"/>
-      <c r="BE43" s="1"/>
-      <c r="BF43" s="1"/>
-      <c r="BG43" s="1"/>
-      <c r="BH43" s="1"/>
-      <c r="BI43" s="1"/>
-      <c r="BJ43" s="1"/>
-      <c r="BK43" s="1"/>
-      <c r="BL43" s="1"/>
-      <c r="BM43" s="1"/>
-      <c r="BN43" s="1"/>
-      <c r="BO43" s="1"/>
-      <c r="BP43" s="1"/>
-      <c r="BQ43" s="1"/>
-      <c r="BR43" s="1"/>
-      <c r="BS43" s="1"/>
-      <c r="BT43" s="1"/>
-      <c r="BU43" s="1"/>
-      <c r="BV43" s="1"/>
-      <c r="BW43" s="1"/>
-      <c r="BX43" s="1"/>
-      <c r="BY43" s="1"/>
-      <c r="BZ43" s="1"/>
-      <c r="CA43" s="1"/>
-      <c r="CB43" s="1"/>
-      <c r="CC43" s="1"/>
-      <c r="CD43" s="1"/>
-      <c r="CE43" s="1"/>
-      <c r="CF43" s="1"/>
-      <c r="CG43" s="1"/>
-      <c r="CH43" s="1"/>
-      <c r="CI43" s="1"/>
-      <c r="CJ43" s="1"/>
-      <c r="CK43" s="1"/>
-      <c r="CL43" s="1"/>
-      <c r="CM43" s="1"/>
-      <c r="CN43" s="1"/>
-      <c r="CO43" s="1"/>
-      <c r="CP43" s="1"/>
-      <c r="CQ43" s="1"/>
-      <c r="CR43" s="1"/>
-      <c r="CS43" s="1"/>
-      <c r="CT43" s="1"/>
-      <c r="CU43" s="1"/>
-      <c r="CV43" s="1"/>
-      <c r="CW43" s="1"/>
-      <c r="CX43" s="1"/>
-      <c r="CY43" s="1"/>
-      <c r="CZ43" s="1"/>
-      <c r="DA43" s="1"/>
-      <c r="DB43" s="1"/>
-      <c r="DC43" s="1"/>
-      <c r="DD43" s="1"/>
-      <c r="DE43" s="1"/>
-      <c r="DF43" s="1"/>
-      <c r="DG43" s="1"/>
-      <c r="DH43" s="1"/>
-      <c r="DI43" s="1"/>
-      <c r="DJ43" s="1"/>
-      <c r="DK43" s="1"/>
-      <c r="DL43" s="1"/>
-      <c r="DM43" s="1"/>
-      <c r="DN43" s="1"/>
-      <c r="DO43" s="1"/>
-      <c r="DP43" s="1"/>
-      <c r="DQ43" s="1"/>
-      <c r="DR43" s="1"/>
-      <c r="DS43" s="1"/>
-      <c r="DT43" s="1"/>
-      <c r="DU43" s="1"/>
-      <c r="DV43" s="1"/>
-      <c r="DW43" s="1"/>
-      <c r="DX43" s="1"/>
-      <c r="DY43" s="1"/>
-      <c r="DZ43" s="1"/>
-      <c r="EA43" s="1"/>
-      <c r="EB43" s="1"/>
-      <c r="EC43" s="1"/>
-      <c r="ED43" s="1"/>
-      <c r="EE43" s="1"/>
-      <c r="EF43" s="1"/>
-      <c r="EG43" s="1"/>
-      <c r="EH43" s="1"/>
-      <c r="EI43" s="1"/>
-      <c r="EJ43" s="1"/>
-      <c r="EK43" s="1"/>
-      <c r="EL43" s="1"/>
-      <c r="EM43" s="1"/>
-      <c r="EN43" s="1"/>
-      <c r="EO43" s="1"/>
-      <c r="EP43" s="1"/>
-      <c r="EQ43" s="1"/>
-      <c r="ER43" s="1"/>
-      <c r="ES43" s="1"/>
-      <c r="ET43" s="1"/>
-      <c r="EU43" s="1"/>
-      <c r="EV43" s="1"/>
-      <c r="EW43" s="1"/>
-      <c r="EX43" s="1"/>
-      <c r="EY43" s="1"/>
-      <c r="EZ43" s="1"/>
-      <c r="FA43" s="1"/>
-      <c r="FB43" s="1"/>
-      <c r="FC43" s="1"/>
-      <c r="FD43" s="1"/>
-      <c r="FE43" s="1"/>
-      <c r="FF43" s="1"/>
-      <c r="FG43" s="1"/>
-      <c r="FH43" s="1"/>
-      <c r="FI43" s="1"/>
-      <c r="FJ43" s="1"/>
-      <c r="FK43" s="1"/>
-      <c r="FL43" s="1"/>
-      <c r="FM43" s="1"/>
-      <c r="FN43" s="1"/>
-      <c r="FO43" s="1"/>
-      <c r="FP43" s="1"/>
-      <c r="FQ43" s="1"/>
-      <c r="FR43" s="1"/>
-      <c r="FS43" s="1"/>
-      <c r="FT43" s="1"/>
-      <c r="FU43" s="1"/>
-      <c r="FV43" s="1"/>
-      <c r="FW43" s="1"/>
-      <c r="FX43" s="1"/>
-      <c r="FY43" s="1"/>
-      <c r="FZ43" s="1"/>
-      <c r="GA43" s="1"/>
-      <c r="GB43" s="1"/>
-      <c r="GC43" s="1"/>
-      <c r="GD43" s="1"/>
-      <c r="GE43" s="1"/>
-      <c r="GF43" s="1"/>
-      <c r="GG43" s="1"/>
-      <c r="GH43" s="1"/>
-      <c r="GI43" s="1"/>
-      <c r="GJ43" s="1"/>
-      <c r="GK43" s="1"/>
-      <c r="GL43" s="1"/>
-      <c r="GM43" s="1"/>
-      <c r="GN43" s="1"/>
-      <c r="GO43" s="1"/>
-      <c r="GP43" s="1"/>
-      <c r="GQ43" s="1"/>
-      <c r="GR43" s="1"/>
-      <c r="GS43" s="1"/>
-      <c r="GT43" s="1"/>
-      <c r="GU43" s="1"/>
-      <c r="GV43" s="1"/>
-      <c r="GW43" s="1"/>
-      <c r="GX43" s="1"/>
-      <c r="GY43" s="1"/>
-      <c r="GZ43" s="1"/>
-      <c r="HA43" s="1"/>
-      <c r="HB43" s="1"/>
-      <c r="HC43" s="1"/>
-      <c r="HD43" s="1"/>
-      <c r="HE43" s="1"/>
-      <c r="HF43" s="1"/>
-      <c r="HG43" s="1"/>
-      <c r="HH43" s="1"/>
-      <c r="HI43" s="1"/>
-      <c r="HJ43" s="1"/>
-      <c r="HK43" s="1"/>
-      <c r="HL43" s="1"/>
-      <c r="HM43" s="1"/>
-      <c r="HN43" s="1"/>
-      <c r="HO43" s="1"/>
-      <c r="HP43" s="1"/>
-      <c r="HQ43" s="1"/>
-      <c r="HR43" s="1"/>
-      <c r="HS43" s="1"/>
-      <c r="HT43" s="1"/>
-      <c r="HU43" s="1"/>
-      <c r="HV43" s="1"/>
-      <c r="HW43" s="1"/>
-      <c r="HX43" s="1"/>
-      <c r="HY43" s="1"/>
-      <c r="HZ43" s="1"/>
-      <c r="IA43" s="1"/>
-      <c r="IB43" s="1"/>
-      <c r="IC43" s="1"/>
-      <c r="ID43" s="1"/>
-      <c r="IE43" s="1"/>
-      <c r="IF43" s="1"/>
-      <c r="IG43" s="1"/>
-      <c r="IH43" s="1"/>
-      <c r="II43" s="1"/>
-      <c r="IJ43" s="1"/>
-      <c r="IK43" s="1"/>
-      <c r="IL43" s="1"/>
-      <c r="IM43" s="1"/>
-      <c r="IN43" s="1"/>
-      <c r="IO43" s="1"/>
-      <c r="IP43" s="1"/>
-      <c r="IQ43" s="1"/>
-      <c r="IR43" s="1"/>
-      <c r="IS43" s="1"/>
-      <c r="IT43" s="1"/>
-      <c r="IU43" s="1"/>
-      <c r="IV43" s="1"/>
+    <row r="43" spans="1:256" ht="14">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
     </row>
-    <row r="44" spans="1:256" s="5" customFormat="1" ht="21" customHeight="1" thickBot="1">
-      <c r="A44" s="6"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="61" t="s">
-        <v>0</v>
-      </c>
-      <c r="D44" s="62"/>
-      <c r="E44" s="62"/>
-      <c r="F44" s="62"/>
-      <c r="G44" s="62"/>
-      <c r="H44" s="63"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="6"/>
-      <c r="K44" s="1"/>
-      <c r="L44" s="1"/>
-      <c r="M44" s="1"/>
-      <c r="N44" s="1"/>
-      <c r="O44" s="1"/>
-      <c r="P44" s="1"/>
-      <c r="Q44" s="1"/>
-      <c r="R44" s="1"/>
-      <c r="S44" s="1"/>
-      <c r="T44" s="1"/>
-      <c r="U44" s="1"/>
-      <c r="V44" s="1"/>
-      <c r="W44" s="1"/>
-      <c r="X44" s="1"/>
-      <c r="Y44" s="1"/>
-      <c r="Z44" s="1"/>
-      <c r="AA44" s="1"/>
-      <c r="AB44" s="1"/>
-      <c r="AC44" s="1"/>
-      <c r="AD44" s="1"/>
-      <c r="AE44" s="1"/>
-      <c r="AF44" s="1"/>
-      <c r="AG44" s="1"/>
-      <c r="AH44" s="1"/>
-      <c r="AI44" s="1"/>
-      <c r="AJ44" s="1"/>
-      <c r="AK44" s="1"/>
-      <c r="AL44" s="1"/>
-      <c r="AM44" s="1"/>
-      <c r="AN44" s="1"/>
-      <c r="AO44" s="1"/>
-      <c r="AP44" s="1"/>
-      <c r="AQ44" s="1"/>
-      <c r="AR44" s="1"/>
-      <c r="AS44" s="1"/>
-      <c r="AT44" s="1"/>
-      <c r="AU44" s="1"/>
-      <c r="AV44" s="1"/>
-      <c r="AW44" s="1"/>
-      <c r="AX44" s="1"/>
-      <c r="AY44" s="1"/>
-      <c r="AZ44" s="1"/>
-      <c r="BA44" s="1"/>
-      <c r="BB44" s="1"/>
-      <c r="BC44" s="1"/>
-      <c r="BD44" s="1"/>
-      <c r="BE44" s="1"/>
-      <c r="BF44" s="1"/>
-      <c r="BG44" s="1"/>
-      <c r="BH44" s="1"/>
-      <c r="BI44" s="1"/>
-      <c r="BJ44" s="1"/>
-      <c r="BK44" s="1"/>
-      <c r="BL44" s="1"/>
-      <c r="BM44" s="1"/>
-      <c r="BN44" s="1"/>
-      <c r="BO44" s="1"/>
-      <c r="BP44" s="1"/>
-      <c r="BQ44" s="1"/>
-      <c r="BR44" s="1"/>
-      <c r="BS44" s="1"/>
-      <c r="BT44" s="1"/>
-      <c r="BU44" s="1"/>
-      <c r="BV44" s="1"/>
-      <c r="BW44" s="1"/>
-      <c r="BX44" s="1"/>
-      <c r="BY44" s="1"/>
-      <c r="BZ44" s="1"/>
-      <c r="CA44" s="1"/>
-      <c r="CB44" s="1"/>
-      <c r="CC44" s="1"/>
-      <c r="CD44" s="1"/>
-      <c r="CE44" s="1"/>
-      <c r="CF44" s="1"/>
-      <c r="CG44" s="1"/>
-      <c r="CH44" s="1"/>
-      <c r="CI44" s="1"/>
-      <c r="CJ44" s="1"/>
-      <c r="CK44" s="1"/>
-      <c r="CL44" s="1"/>
-      <c r="CM44" s="1"/>
-      <c r="CN44" s="1"/>
-      <c r="CO44" s="1"/>
-      <c r="CP44" s="1"/>
-      <c r="CQ44" s="1"/>
-      <c r="CR44" s="1"/>
-      <c r="CS44" s="1"/>
-      <c r="CT44" s="1"/>
-      <c r="CU44" s="1"/>
-      <c r="CV44" s="1"/>
-      <c r="CW44" s="1"/>
-      <c r="CX44" s="1"/>
-      <c r="CY44" s="1"/>
-      <c r="CZ44" s="1"/>
-      <c r="DA44" s="1"/>
-      <c r="DB44" s="1"/>
-      <c r="DC44" s="1"/>
-      <c r="DD44" s="1"/>
-      <c r="DE44" s="1"/>
-      <c r="DF44" s="1"/>
-      <c r="DG44" s="1"/>
-      <c r="DH44" s="1"/>
-      <c r="DI44" s="1"/>
-      <c r="DJ44" s="1"/>
-      <c r="DK44" s="1"/>
-      <c r="DL44" s="1"/>
-      <c r="DM44" s="1"/>
-      <c r="DN44" s="1"/>
-      <c r="DO44" s="1"/>
-      <c r="DP44" s="1"/>
-      <c r="DQ44" s="1"/>
-      <c r="DR44" s="1"/>
-      <c r="DS44" s="1"/>
-      <c r="DT44" s="1"/>
-      <c r="DU44" s="1"/>
-      <c r="DV44" s="1"/>
-      <c r="DW44" s="1"/>
-      <c r="DX44" s="1"/>
-      <c r="DY44" s="1"/>
-      <c r="DZ44" s="1"/>
-      <c r="EA44" s="1"/>
-      <c r="EB44" s="1"/>
-      <c r="EC44" s="1"/>
-      <c r="ED44" s="1"/>
-      <c r="EE44" s="1"/>
-      <c r="EF44" s="1"/>
-      <c r="EG44" s="1"/>
-      <c r="EH44" s="1"/>
-      <c r="EI44" s="1"/>
-      <c r="EJ44" s="1"/>
-      <c r="EK44" s="1"/>
-      <c r="EL44" s="1"/>
-      <c r="EM44" s="1"/>
-      <c r="EN44" s="1"/>
-      <c r="EO44" s="1"/>
-      <c r="EP44" s="1"/>
-      <c r="EQ44" s="1"/>
-      <c r="ER44" s="1"/>
-      <c r="ES44" s="1"/>
-      <c r="ET44" s="1"/>
-      <c r="EU44" s="1"/>
-      <c r="EV44" s="1"/>
-      <c r="EW44" s="1"/>
-      <c r="EX44" s="1"/>
-      <c r="EY44" s="1"/>
-      <c r="EZ44" s="1"/>
-      <c r="FA44" s="1"/>
-      <c r="FB44" s="1"/>
-      <c r="FC44" s="1"/>
-      <c r="FD44" s="1"/>
-      <c r="FE44" s="1"/>
-      <c r="FF44" s="1"/>
-      <c r="FG44" s="1"/>
-      <c r="FH44" s="1"/>
-      <c r="FI44" s="1"/>
-      <c r="FJ44" s="1"/>
-      <c r="FK44" s="1"/>
-      <c r="FL44" s="1"/>
-      <c r="FM44" s="1"/>
-      <c r="FN44" s="1"/>
-      <c r="FO44" s="1"/>
-      <c r="FP44" s="1"/>
-      <c r="FQ44" s="1"/>
-      <c r="FR44" s="1"/>
-      <c r="FS44" s="1"/>
-      <c r="FT44" s="1"/>
-      <c r="FU44" s="1"/>
-      <c r="FV44" s="1"/>
-      <c r="FW44" s="1"/>
-      <c r="FX44" s="1"/>
-      <c r="FY44" s="1"/>
-      <c r="FZ44" s="1"/>
-      <c r="GA44" s="1"/>
-      <c r="GB44" s="1"/>
-      <c r="GC44" s="1"/>
-      <c r="GD44" s="1"/>
-      <c r="GE44" s="1"/>
-      <c r="GF44" s="1"/>
-      <c r="GG44" s="1"/>
-      <c r="GH44" s="1"/>
-      <c r="GI44" s="1"/>
-      <c r="GJ44" s="1"/>
-      <c r="GK44" s="1"/>
-      <c r="GL44" s="1"/>
-      <c r="GM44" s="1"/>
-      <c r="GN44" s="1"/>
-      <c r="GO44" s="1"/>
-      <c r="GP44" s="1"/>
-      <c r="GQ44" s="1"/>
-      <c r="GR44" s="1"/>
-      <c r="GS44" s="1"/>
-      <c r="GT44" s="1"/>
-      <c r="GU44" s="1"/>
-      <c r="GV44" s="1"/>
-      <c r="GW44" s="1"/>
-      <c r="GX44" s="1"/>
-      <c r="GY44" s="1"/>
-      <c r="GZ44" s="1"/>
-      <c r="HA44" s="1"/>
-      <c r="HB44" s="1"/>
-      <c r="HC44" s="1"/>
-      <c r="HD44" s="1"/>
-      <c r="HE44" s="1"/>
-      <c r="HF44" s="1"/>
-      <c r="HG44" s="1"/>
-      <c r="HH44" s="1"/>
-      <c r="HI44" s="1"/>
-      <c r="HJ44" s="1"/>
-      <c r="HK44" s="1"/>
-      <c r="HL44" s="1"/>
-      <c r="HM44" s="1"/>
-      <c r="HN44" s="1"/>
-      <c r="HO44" s="1"/>
-      <c r="HP44" s="1"/>
-      <c r="HQ44" s="1"/>
-      <c r="HR44" s="1"/>
-      <c r="HS44" s="1"/>
-      <c r="HT44" s="1"/>
-      <c r="HU44" s="1"/>
-      <c r="HV44" s="1"/>
-      <c r="HW44" s="1"/>
-      <c r="HX44" s="1"/>
-      <c r="HY44" s="1"/>
-      <c r="HZ44" s="1"/>
-      <c r="IA44" s="1"/>
-      <c r="IB44" s="1"/>
-      <c r="IC44" s="1"/>
-      <c r="ID44" s="1"/>
-      <c r="IE44" s="1"/>
-      <c r="IF44" s="1"/>
-      <c r="IG44" s="1"/>
-      <c r="IH44" s="1"/>
-      <c r="II44" s="1"/>
-      <c r="IJ44" s="1"/>
-      <c r="IK44" s="1"/>
-      <c r="IL44" s="1"/>
-      <c r="IM44" s="1"/>
-      <c r="IN44" s="1"/>
-      <c r="IO44" s="1"/>
-      <c r="IP44" s="1"/>
-      <c r="IQ44" s="1"/>
-      <c r="IR44" s="1"/>
-      <c r="IS44" s="1"/>
-      <c r="IT44" s="1"/>
-      <c r="IU44" s="1"/>
-      <c r="IV44" s="1"/>
-    </row>
-    <row r="45" spans="1:256" ht="14.25">
-      <c r="A45" s="3"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="3"/>
-    </row>
-    <row r="46" spans="1:256" ht="14.25">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
-      <c r="J46" s="3"/>
-    </row>
-    <row r="48" spans="1:256" ht="14.25">
-      <c r="H48" s="2"/>
+    <row r="45" spans="1:256" ht="14">
+      <c r="H45" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C32:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="C3:D7"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="F7:H7"/>
-    <mergeCell ref="C15:H15"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="C35:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="C42:H42"/>
-    <mergeCell ref="C43:H43"/>
-    <mergeCell ref="C44:H44"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="C9:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>